<commit_message>
Rilascio V_S_12.10.1.0 2026-08-28 (Patch Mesi di Aprile, Maggio, Giugno, Luglio e Agosto 2026)
</commit_message>
<xml_diff>
--- a/RILASCIO_12.9.2.0/SIUT-SIES-CT-1.0-20260327-Allegato_al_piano_test_SIES_v.12.9.2.0.xlsx
+++ b/RILASCIO_12.9.2.0/SIUT-SIES-CT-1.0-20260327-Allegato_al_piano_test_SIES_v.12.9.2.0.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView xWindow="-15" yWindow="-15" windowWidth="20520" windowHeight="9360" tabRatio="795" firstSheet="3" activeTab="3"/>
+    <workbookView xWindow="-15" yWindow="-15" windowWidth="20520" windowHeight="9360" tabRatio="795" firstSheet="3" activeTab="9"/>
   </bookViews>
   <sheets>
     <sheet name="Raw_Data_In" sheetId="703" state="hidden" r:id="rId1"/>
@@ -5555,6 +5555,33 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="11" borderId="57" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="76" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="57" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="74" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="77" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="78" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="74" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="77" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="78" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -5589,33 +5616,6 @@
     <xf numFmtId="0" fontId="8" fillId="12" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="11" borderId="57" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="76" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="57" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="74" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="77" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="78" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="74" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="77" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="78" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -5654,6 +5654,21 @@
     <xf numFmtId="0" fontId="23" fillId="3" borderId="81" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="75" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="79" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="45" fillId="2" borderId="82" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -5719,21 +5734,6 @@
     </xf>
     <xf numFmtId="0" fontId="52" fillId="2" borderId="90" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="75" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="79" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="75" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -5761,6 +5761,15 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="8" fillId="11" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="11" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -5768,18 +5777,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="38" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="38" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="11" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="11" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="37" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -5835,69 +5832,57 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="38" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="18" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="80" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="12" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="4" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="80" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="14" fillId="16" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="16" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="67" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -5910,26 +5895,41 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="80" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="4" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="15" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="80" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="14" fillId="16" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="16" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="49" fontId="26" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -5939,42 +5939,6 @@
     </xf>
     <xf numFmtId="165" fontId="26" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="12" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="12" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="75" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -6028,6 +5992,42 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -6092,7 +6092,7 @@
 </file>
 
 <file path=xl/activeX/activeX13.xml><?xml version="1.0" encoding="utf-8"?>
-<ax:ocx xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ax:classid="{D7053240-CE69-11CD-A777-00DD01143C57}" ax:persistence="persistStreamInit" r:id="rId1"/>
+<ax:ocx xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ax:classid="{8BD21D50-EC42-11CE-9E0D-00AA006002F3}" ax:persistence="persistStreamInit" r:id="rId1"/>
 </file>
 
 <file path=xl/activeX/activeX14.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6112,7 +6112,7 @@
 </file>
 
 <file path=xl/activeX/activeX18.xml><?xml version="1.0" encoding="utf-8"?>
-<ax:ocx xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ax:classid="{8BD21D50-EC42-11CE-9E0D-00AA006002F3}" ax:persistence="persistStreamInit" r:id="rId1"/>
+<ax:ocx xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ax:classid="{D7053240-CE69-11CD-A777-00DD01143C57}" ax:persistence="persistStreamInit" r:id="rId1"/>
 </file>
 
 <file path=xl/activeX/activeX2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9695,38 +9695,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="30" customHeight="1" thickBot="1">
-      <c r="A1" s="395" t="s">
+      <c r="A1" s="404" t="s">
         <v>212</v>
       </c>
-      <c r="B1" s="396"/>
-      <c r="C1" s="397"/>
-      <c r="D1" s="389" t="str">
+      <c r="B1" s="405"/>
+      <c r="C1" s="406"/>
+      <c r="D1" s="398" t="str">
         <f>Copertina!C7</f>
         <v>SIES v.12.9.2.0</v>
       </c>
-      <c r="E1" s="390"/>
-      <c r="F1" s="390"/>
-      <c r="G1" s="390"/>
-      <c r="H1" s="390"/>
-      <c r="I1" s="390"/>
-      <c r="J1" s="391"/>
+      <c r="E1" s="399"/>
+      <c r="F1" s="399"/>
+      <c r="G1" s="399"/>
+      <c r="H1" s="399"/>
+      <c r="I1" s="399"/>
+      <c r="J1" s="400"/>
     </row>
     <row r="2" spans="1:10" ht="30" customHeight="1" thickBot="1">
-      <c r="A2" s="395" t="s">
+      <c r="A2" s="404" t="s">
         <v>74</v>
       </c>
-      <c r="B2" s="396"/>
-      <c r="C2" s="398"/>
-      <c r="D2" s="392" t="str">
+      <c r="B2" s="405"/>
+      <c r="C2" s="407"/>
+      <c r="D2" s="401" t="str">
         <f>Copertina!C3</f>
         <v>SIUT-SIES-CT-1.0-20260327-Allegato_al_piano_test_SIES_v.12.9.2.0.xlsx</v>
       </c>
-      <c r="E2" s="393"/>
-      <c r="F2" s="393"/>
-      <c r="G2" s="393"/>
-      <c r="H2" s="393"/>
-      <c r="I2" s="393"/>
-      <c r="J2" s="394"/>
+      <c r="E2" s="402"/>
+      <c r="F2" s="402"/>
+      <c r="G2" s="402"/>
+      <c r="H2" s="402"/>
+      <c r="I2" s="402"/>
+      <c r="J2" s="403"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" thickBot="1">
       <c r="A3" s="301" t="s">
@@ -9735,14 +9735,14 @@
       <c r="B3" s="302" t="s">
         <v>588</v>
       </c>
-      <c r="C3" s="399" t="s">
+      <c r="C3" s="408" t="s">
         <v>589</v>
       </c>
-      <c r="D3" s="399"/>
-      <c r="E3" s="399" t="s">
+      <c r="D3" s="408"/>
+      <c r="E3" s="408" t="s">
         <v>185</v>
       </c>
-      <c r="F3" s="399"/>
+      <c r="F3" s="408"/>
       <c r="G3" s="303" t="s">
         <v>174</v>
       </c>
@@ -9765,16 +9765,16 @@
         <f>TabellaTest!I4</f>
         <v>SIEP</v>
       </c>
-      <c r="C4" s="400" t="str">
+      <c r="C4" s="389" t="str">
         <f>TabellaTest!L4</f>
         <v>Errore inserimento dati con apostrofo</v>
       </c>
-      <c r="D4" s="401"/>
-      <c r="E4" s="402" t="str">
+      <c r="D4" s="390"/>
+      <c r="E4" s="391" t="str">
         <f>TabellaTest!P4</f>
         <v>Verifica: Verificare il corretto inserimento di nome, cognome o comune contenenti un apostrofo</v>
       </c>
-      <c r="F4" s="401"/>
+      <c r="F4" s="390"/>
       <c r="G4" s="318" t="str">
         <f>TabellaTest!Q4</f>
         <v>1.0</v>
@@ -9784,7 +9784,7 @@
       <c r="J4" s="318"/>
     </row>
     <row r="5" spans="1:10" s="332" customFormat="1" ht="30" customHeight="1">
-      <c r="A5" s="403"/>
+      <c r="A5" s="392"/>
       <c r="B5" s="319" t="s">
         <v>188</v>
       </c>
@@ -9800,13 +9800,13 @@
       <c r="F5" s="349" t="s">
         <v>598</v>
       </c>
-      <c r="G5" s="403"/>
+      <c r="G5" s="392"/>
       <c r="H5" s="321"/>
       <c r="I5" s="321"/>
-      <c r="J5" s="406"/>
+      <c r="J5" s="395"/>
     </row>
     <row r="6" spans="1:10" s="332" customFormat="1" ht="45" customHeight="1">
-      <c r="A6" s="404"/>
+      <c r="A6" s="393"/>
       <c r="B6" s="337" t="s">
         <v>164</v>
       </c>
@@ -9820,13 +9820,13 @@
         <v>625</v>
       </c>
       <c r="F6" s="350"/>
-      <c r="G6" s="404"/>
+      <c r="G6" s="393"/>
       <c r="H6" s="333"/>
       <c r="I6" s="333"/>
-      <c r="J6" s="407"/>
+      <c r="J6" s="396"/>
     </row>
     <row r="7" spans="1:10" s="332" customFormat="1" ht="45" customHeight="1">
-      <c r="A7" s="404"/>
+      <c r="A7" s="393"/>
       <c r="B7" s="337" t="s">
         <v>164</v>
       </c>
@@ -9842,13 +9842,13 @@
       <c r="F7" s="352" t="s">
         <v>619</v>
       </c>
-      <c r="G7" s="404"/>
+      <c r="G7" s="393"/>
       <c r="H7" s="333"/>
       <c r="I7" s="333"/>
-      <c r="J7" s="407"/>
+      <c r="J7" s="396"/>
     </row>
     <row r="8" spans="1:10" s="332" customFormat="1" ht="30" customHeight="1">
-      <c r="A8" s="404"/>
+      <c r="A8" s="393"/>
       <c r="B8" s="341">
         <v>1</v>
       </c>
@@ -9864,13 +9864,13 @@
       <c r="F8" s="350" t="s">
         <v>620</v>
       </c>
-      <c r="G8" s="404"/>
+      <c r="G8" s="393"/>
       <c r="H8" s="333"/>
       <c r="I8" s="333"/>
-      <c r="J8" s="407"/>
+      <c r="J8" s="396"/>
     </row>
     <row r="9" spans="1:10" s="335" customFormat="1" ht="30" customHeight="1">
-      <c r="A9" s="404"/>
+      <c r="A9" s="393"/>
       <c r="B9" s="344">
         <v>2</v>
       </c>
@@ -9884,13 +9884,13 @@
       <c r="F9" s="350" t="s">
         <v>614</v>
       </c>
-      <c r="G9" s="404"/>
+      <c r="G9" s="393"/>
       <c r="H9" s="336"/>
       <c r="I9" s="336"/>
-      <c r="J9" s="407"/>
+      <c r="J9" s="396"/>
     </row>
     <row r="10" spans="1:10" s="332" customFormat="1" ht="30" customHeight="1">
-      <c r="A10" s="404"/>
+      <c r="A10" s="393"/>
       <c r="B10" s="344">
         <v>3</v>
       </c>
@@ -9904,13 +9904,13 @@
       <c r="F10" s="350" t="s">
         <v>617</v>
       </c>
-      <c r="G10" s="404"/>
+      <c r="G10" s="393"/>
       <c r="H10" s="333"/>
       <c r="I10" s="333"/>
-      <c r="J10" s="407"/>
+      <c r="J10" s="396"/>
     </row>
     <row r="11" spans="1:10" ht="60" customHeight="1" thickBot="1">
-      <c r="A11" s="405"/>
+      <c r="A11" s="394"/>
       <c r="B11" s="346" t="s">
         <v>199</v>
       </c>
@@ -9924,22 +9924,22 @@
       <c r="F11" s="351" t="s">
         <v>623</v>
       </c>
-      <c r="G11" s="405"/>
-      <c r="J11" s="408"/>
+      <c r="G11" s="394"/>
+      <c r="J11" s="397"/>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="A5:A11"/>
-    <mergeCell ref="G5:G11"/>
-    <mergeCell ref="J5:J11"/>
     <mergeCell ref="D1:J1"/>
     <mergeCell ref="D2:J2"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="E3:F3"/>
     <mergeCell ref="C3:D3"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="A5:A11"/>
+    <mergeCell ref="G5:G11"/>
+    <mergeCell ref="J5:J11"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.27559055118110237" right="0.55118110236220474" top="0.43307086614173229" bottom="0.39370078740157483" header="0.23622047244094491" footer="0.23622047244094491"/>
@@ -9953,27 +9953,27 @@
   <controls>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="260100" r:id="rId4" name="Btn_InsLayout">
+        <control shapeId="260103" r:id="rId4" name="Btn_Duplicate">
           <controlPr defaultSize="0" print="0" autoLine="0" r:id="rId5">
             <anchor>
               <from>
-                <xdr:col>3</xdr:col>
-                <xdr:colOff>381000</xdr:colOff>
+                <xdr:col>4</xdr:col>
+                <xdr:colOff>771525</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>9525</xdr:rowOff>
               </from>
               <to>
-                <xdr:col>3</xdr:col>
-                <xdr:colOff>2057400</xdr:colOff>
+                <xdr:col>4</xdr:col>
+                <xdr:colOff>1895475</xdr:colOff>
                 <xdr:row>0</xdr:row>
-                <xdr:rowOff>361950</xdr:rowOff>
+                <xdr:rowOff>371475</xdr:rowOff>
               </to>
             </anchor>
           </controlPr>
         </control>
       </mc:Choice>
       <mc:Fallback>
-        <control shapeId="260100" r:id="rId4" name="Btn_InsLayout"/>
+        <control shapeId="260103" r:id="rId4" name="Btn_Duplicate"/>
       </mc:Fallback>
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -10003,27 +10003,27 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="260103" r:id="rId8" name="Btn_Duplicate">
+        <control shapeId="260100" r:id="rId8" name="Btn_InsLayout">
           <controlPr defaultSize="0" print="0" autoLine="0" r:id="rId9">
             <anchor>
               <from>
-                <xdr:col>4</xdr:col>
-                <xdr:colOff>771525</xdr:colOff>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>381000</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>9525</xdr:rowOff>
               </from>
               <to>
-                <xdr:col>4</xdr:col>
-                <xdr:colOff>1895475</xdr:colOff>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>2057400</xdr:colOff>
                 <xdr:row>0</xdr:row>
-                <xdr:rowOff>371475</xdr:rowOff>
+                <xdr:rowOff>361950</xdr:rowOff>
               </to>
             </anchor>
           </controlPr>
         </control>
       </mc:Choice>
       <mc:Fallback>
-        <control shapeId="260103" r:id="rId8" name="Btn_Duplicate"/>
+        <control shapeId="260100" r:id="rId8" name="Btn_InsLayout"/>
       </mc:Fallback>
     </mc:AlternateContent>
   </controls>
@@ -10046,7 +10046,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" s="88" customFormat="1" ht="21" thickBot="1">
-      <c r="A1" s="395" t="s">
+      <c r="A1" s="404" t="s">
         <v>212</v>
       </c>
       <c r="B1" s="409"/>
@@ -10207,59 +10207,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="16.5" customHeight="1" thickBot="1">
-      <c r="A1" s="395" t="s">
+      <c r="A1" s="404" t="s">
         <v>212</v>
       </c>
       <c r="B1" s="409"/>
       <c r="C1" s="409"/>
-      <c r="D1" s="442" t="str">
+      <c r="D1" s="420" t="str">
         <f>VerificheConformità!E1</f>
         <v>Intervento</v>
       </c>
-      <c r="E1" s="443"/>
+      <c r="E1" s="421"/>
     </row>
     <row r="2" spans="1:9" ht="21" customHeight="1" thickBot="1">
-      <c r="A2" s="395" t="s">
+      <c r="A2" s="404" t="s">
         <v>74</v>
       </c>
       <c r="B2" s="409"/>
       <c r="C2" s="409"/>
-      <c r="D2" s="442" t="e">
+      <c r="D2" s="420" t="e">
         <f>VerificheConformità!E2</f>
         <v>#REF!</v>
       </c>
-      <c r="E2" s="443"/>
+      <c r="E2" s="421"/>
     </row>
     <row r="3" spans="1:9" s="88" customFormat="1" ht="27" customHeight="1" thickBot="1">
-      <c r="A3" s="425" t="s">
+      <c r="A3" s="430" t="s">
         <v>583</v>
       </c>
-      <c r="B3" s="426"/>
-      <c r="C3" s="426"/>
-      <c r="D3" s="427"/>
-      <c r="E3" s="428"/>
-      <c r="G3" s="429" t="s">
+      <c r="B3" s="431"/>
+      <c r="C3" s="431"/>
+      <c r="D3" s="432"/>
+      <c r="E3" s="433"/>
+      <c r="G3" s="434" t="s">
         <v>584</v>
       </c>
-      <c r="H3" s="430"/>
-      <c r="I3" s="431"/>
+      <c r="H3" s="435"/>
+      <c r="I3" s="436"/>
     </row>
     <row r="4" spans="1:9" ht="23.25" customHeight="1" thickBot="1">
-      <c r="A4" s="438" t="s">
+      <c r="A4" s="443" t="s">
         <v>585</v>
       </c>
-      <c r="B4" s="439" t="s">
+      <c r="B4" s="444" t="s">
         <v>586</v>
       </c>
-      <c r="C4" s="440"/>
-      <c r="D4" s="440"/>
-      <c r="E4" s="441"/>
-      <c r="G4" s="432"/>
-      <c r="H4" s="433"/>
-      <c r="I4" s="434"/>
+      <c r="C4" s="445"/>
+      <c r="D4" s="445"/>
+      <c r="E4" s="446"/>
+      <c r="G4" s="437"/>
+      <c r="H4" s="438"/>
+      <c r="I4" s="439"/>
     </row>
     <row r="5" spans="1:9" ht="26.25" customHeight="1" thickBot="1">
-      <c r="A5" s="421"/>
+      <c r="A5" s="426"/>
       <c r="B5" s="269">
         <v>1</v>
       </c>
@@ -10272,9 +10272,9 @@
       <c r="E5" s="270">
         <v>4</v>
       </c>
-      <c r="G5" s="432"/>
-      <c r="H5" s="433"/>
-      <c r="I5" s="434"/>
+      <c r="G5" s="437"/>
+      <c r="H5" s="438"/>
+      <c r="I5" s="439"/>
     </row>
     <row r="6" spans="1:9" ht="15.75" thickBot="1">
       <c r="A6" s="271" t="s">
@@ -10296,9 +10296,9 @@
         <f>COUNTIFS(TabellaTest!M4:M269,4,TabellaTest!T4:T269,"A",TabellaTest!U4:U269,"KO")</f>
         <v>0</v>
       </c>
-      <c r="G6" s="432"/>
-      <c r="H6" s="433"/>
-      <c r="I6" s="434"/>
+      <c r="G6" s="437"/>
+      <c r="H6" s="438"/>
+      <c r="I6" s="439"/>
     </row>
     <row r="7" spans="1:9" ht="15.75" thickBot="1">
       <c r="A7" s="273" t="s">
@@ -10320,9 +10320,9 @@
         <f>COUNTIFS(TabellaTest!M4:M269,4,TabellaTest!T4:T269,"B",TabellaTest!U4:U269,"KO")</f>
         <v>0</v>
       </c>
-      <c r="G7" s="432"/>
-      <c r="H7" s="433"/>
-      <c r="I7" s="434"/>
+      <c r="G7" s="437"/>
+      <c r="H7" s="438"/>
+      <c r="I7" s="439"/>
     </row>
     <row r="8" spans="1:9" ht="15.75" thickBot="1">
       <c r="A8" s="274" t="s">
@@ -10344,9 +10344,9 @@
         <f>COUNTIFS(TabellaTest!M4:M269,4,TabellaTest!T4:T269,"C",TabellaTest!U4:U269,"KO")</f>
         <v>0</v>
       </c>
-      <c r="G8" s="435"/>
-      <c r="H8" s="436"/>
-      <c r="I8" s="437"/>
+      <c r="G8" s="440"/>
+      <c r="H8" s="441"/>
+      <c r="I8" s="442"/>
     </row>
     <row r="9" spans="1:9">
       <c r="G9" s="267"/>
@@ -10356,27 +10356,27 @@
     <row r="12" spans="1:9" ht="10.5" customHeight="1" thickBot="1"/>
     <row r="13" spans="1:9" ht="13.5" hidden="1" thickBot="1"/>
     <row r="14" spans="1:9" s="88" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A14" s="444" t="s">
+      <c r="A14" s="422" t="s">
         <v>587</v>
       </c>
-      <c r="B14" s="445"/>
-      <c r="C14" s="445"/>
-      <c r="D14" s="445"/>
-      <c r="E14" s="446"/>
+      <c r="B14" s="423"/>
+      <c r="C14" s="423"/>
+      <c r="D14" s="423"/>
+      <c r="E14" s="424"/>
     </row>
     <row r="15" spans="1:9" ht="15.75" thickBot="1">
-      <c r="A15" s="420" t="s">
+      <c r="A15" s="425" t="s">
         <v>585</v>
       </c>
-      <c r="B15" s="422" t="s">
+      <c r="B15" s="427" t="s">
         <v>586</v>
       </c>
-      <c r="C15" s="423"/>
-      <c r="D15" s="423"/>
-      <c r="E15" s="424"/>
+      <c r="C15" s="428"/>
+      <c r="D15" s="428"/>
+      <c r="E15" s="429"/>
     </row>
     <row r="16" spans="1:9" ht="15" thickBot="1">
-      <c r="A16" s="421"/>
+      <c r="A16" s="426"/>
       <c r="B16" s="275">
         <v>1</v>
       </c>
@@ -10456,17 +10456,17 @@
   </sheetData>
   <sheetProtection password="A7EC" sheet="1" objects="1" scenarios="1" selectLockedCells="1" selectUnlockedCells="1"/>
   <mergeCells count="11">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="A14:E14"/>
     <mergeCell ref="A15:A16"/>
     <mergeCell ref="B15:E15"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="G3:I8"/>
     <mergeCell ref="A4:A5"/>
     <mergeCell ref="B4:E4"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="A14:E14"/>
   </mergeCells>
   <phoneticPr fontId="54" type="noConversion"/>
   <conditionalFormatting sqref="B6:B8">
@@ -10591,34 +10591,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="54.75" customHeight="1">
-      <c r="A1" s="466" t="s">
+      <c r="A1" s="465" t="s">
         <v>212</v>
       </c>
-      <c r="B1" s="467"/>
-      <c r="C1" s="468"/>
-      <c r="D1" s="462" t="s">
+      <c r="B1" s="466"/>
+      <c r="C1" s="467"/>
+      <c r="D1" s="461" t="s">
         <v>334</v>
       </c>
-      <c r="E1" s="463"/>
-      <c r="F1" s="463"/>
-      <c r="G1" s="463"/>
-      <c r="H1" s="464"/>
-      <c r="I1" s="465"/>
+      <c r="E1" s="462"/>
+      <c r="F1" s="462"/>
+      <c r="G1" s="462"/>
+      <c r="H1" s="463"/>
+      <c r="I1" s="464"/>
     </row>
     <row r="2" spans="1:9" ht="22.5" customHeight="1" thickBot="1">
-      <c r="A2" s="469" t="s">
+      <c r="A2" s="468" t="s">
         <v>74</v>
       </c>
-      <c r="B2" s="470"/>
-      <c r="C2" s="471"/>
-      <c r="D2" s="475" t="s">
+      <c r="B2" s="469"/>
+      <c r="C2" s="470"/>
+      <c r="D2" s="474" t="s">
         <v>336</v>
       </c>
-      <c r="E2" s="476"/>
-      <c r="F2" s="477"/>
-      <c r="G2" s="477"/>
-      <c r="H2" s="477"/>
-      <c r="I2" s="478"/>
+      <c r="E2" s="475"/>
+      <c r="F2" s="476"/>
+      <c r="G2" s="476"/>
+      <c r="H2" s="476"/>
+      <c r="I2" s="477"/>
     </row>
     <row r="3" spans="1:9" ht="52.5" customHeight="1">
       <c r="A3" s="72" t="s">
@@ -10627,14 +10627,14 @@
       <c r="B3" s="36" t="s">
         <v>62</v>
       </c>
-      <c r="C3" s="472" t="s">
+      <c r="C3" s="471" t="s">
         <v>61</v>
       </c>
-      <c r="D3" s="473"/>
-      <c r="E3" s="472" t="s">
+      <c r="D3" s="472"/>
+      <c r="E3" s="471" t="s">
         <v>185</v>
       </c>
-      <c r="F3" s="474"/>
+      <c r="F3" s="473"/>
       <c r="G3" s="144" t="s">
         <v>174</v>
       </c>
@@ -10652,14 +10652,14 @@
       <c r="B4" s="188" t="s">
         <v>75</v>
       </c>
-      <c r="C4" s="458" t="s">
+      <c r="C4" s="478" t="s">
         <v>497</v>
       </c>
-      <c r="D4" s="459"/>
-      <c r="E4" s="457" t="s">
+      <c r="D4" s="479"/>
+      <c r="E4" s="460" t="s">
         <v>498</v>
       </c>
-      <c r="F4" s="456"/>
+      <c r="F4" s="459"/>
       <c r="G4" s="189"/>
       <c r="H4" s="131"/>
       <c r="I4" s="190"/>
@@ -10839,14 +10839,14 @@
       <c r="B13" s="188" t="s">
         <v>75</v>
       </c>
-      <c r="C13" s="460" t="s">
+      <c r="C13" s="455" t="s">
         <v>344</v>
       </c>
-      <c r="D13" s="461"/>
-      <c r="E13" s="460" t="s">
+      <c r="D13" s="456"/>
+      <c r="E13" s="455" t="s">
         <v>345</v>
       </c>
-      <c r="F13" s="461"/>
+      <c r="F13" s="456"/>
       <c r="G13" s="194" t="s">
         <v>337</v>
       </c>
@@ -11153,15 +11153,15 @@
       <c r="B28" s="188" t="s">
         <v>75</v>
       </c>
-      <c r="C28" s="455" t="str">
+      <c r="C28" s="458" t="str">
         <f>Es.1!L6</f>
         <v>Inserimento dati duplicati</v>
       </c>
-      <c r="D28" s="456"/>
-      <c r="E28" s="457" t="s">
+      <c r="D28" s="459"/>
+      <c r="E28" s="460" t="s">
         <v>498</v>
       </c>
-      <c r="F28" s="456"/>
+      <c r="F28" s="459"/>
       <c r="G28" s="189"/>
       <c r="H28" s="131"/>
       <c r="I28" s="190"/>
@@ -11174,15 +11174,15 @@
       <c r="B29" s="188" t="s">
         <v>75</v>
       </c>
-      <c r="C29" s="455" t="str">
+      <c r="C29" s="458" t="str">
         <f>Es.1!L7</f>
         <v>Inserimento dati non validi</v>
       </c>
-      <c r="D29" s="456"/>
-      <c r="E29" s="457" t="s">
+      <c r="D29" s="459"/>
+      <c r="E29" s="460" t="s">
         <v>498</v>
       </c>
-      <c r="F29" s="456"/>
+      <c r="F29" s="459"/>
       <c r="G29" s="189"/>
       <c r="H29" s="131"/>
       <c r="I29" s="190"/>
@@ -11195,15 +11195,15 @@
       <c r="B30" s="188" t="s">
         <v>75</v>
       </c>
-      <c r="C30" s="455" t="str">
+      <c r="C30" s="458" t="str">
         <f>Es.1!L8</f>
         <v>Verifica Accessibilità</v>
       </c>
-      <c r="D30" s="456"/>
-      <c r="E30" s="457" t="s">
+      <c r="D30" s="459"/>
+      <c r="E30" s="460" t="s">
         <v>498</v>
       </c>
-      <c r="F30" s="456"/>
+      <c r="F30" s="459"/>
       <c r="G30" s="189"/>
       <c r="H30" s="131"/>
       <c r="I30" s="190"/>
@@ -11216,15 +11216,15 @@
       <c r="B31" s="188" t="s">
         <v>75</v>
       </c>
-      <c r="C31" s="455" t="str">
+      <c r="C31" s="458" t="str">
         <f>Es.1!L9</f>
         <v>Verifica Usabilità</v>
       </c>
-      <c r="D31" s="456"/>
-      <c r="E31" s="457" t="s">
+      <c r="D31" s="459"/>
+      <c r="E31" s="460" t="s">
         <v>498</v>
       </c>
-      <c r="F31" s="456"/>
+      <c r="F31" s="459"/>
       <c r="G31" s="189"/>
       <c r="H31" s="131"/>
       <c r="I31" s="190"/>
@@ -11237,15 +11237,15 @@
       <c r="B32" s="188" t="s">
         <v>75</v>
       </c>
-      <c r="C32" s="455" t="str">
+      <c r="C32" s="458" t="str">
         <f>Es.1!L10</f>
         <v>Ricerca - visualizzazione - modifica e cancellazione anagrafica</v>
       </c>
-      <c r="D32" s="456"/>
-      <c r="E32" s="457" t="s">
+      <c r="D32" s="459"/>
+      <c r="E32" s="460" t="s">
         <v>498</v>
       </c>
-      <c r="F32" s="456"/>
+      <c r="F32" s="459"/>
       <c r="G32" s="189"/>
       <c r="H32" s="131"/>
       <c r="I32" s="190"/>
@@ -11258,15 +11258,15 @@
       <c r="B33" s="188" t="s">
         <v>75</v>
       </c>
-      <c r="C33" s="455" t="str">
+      <c r="C33" s="458" t="str">
         <f>Es.1!L11</f>
         <v>Creazione progetto, inserimento e modifica anagrafica, stampa resoconto.</v>
       </c>
-      <c r="D33" s="456"/>
-      <c r="E33" s="457" t="s">
+      <c r="D33" s="459"/>
+      <c r="E33" s="460" t="s">
         <v>498</v>
       </c>
-      <c r="F33" s="456"/>
+      <c r="F33" s="459"/>
       <c r="G33" s="189"/>
       <c r="H33" s="131"/>
       <c r="I33" s="190"/>
@@ -11279,15 +11279,15 @@
       <c r="B34" s="188" t="s">
         <v>75</v>
       </c>
-      <c r="C34" s="455" t="str">
+      <c r="C34" s="458" t="str">
         <f>Es.1!L12</f>
         <v>Ricerca - visualizzazione elenco progetti</v>
       </c>
-      <c r="D34" s="456"/>
-      <c r="E34" s="457" t="s">
+      <c r="D34" s="459"/>
+      <c r="E34" s="460" t="s">
         <v>498</v>
       </c>
-      <c r="F34" s="456"/>
+      <c r="F34" s="459"/>
       <c r="G34" s="189"/>
       <c r="H34" s="131"/>
       <c r="I34" s="190"/>
@@ -11300,15 +11300,15 @@
       <c r="B35" s="188" t="s">
         <v>75</v>
       </c>
-      <c r="C35" s="455" t="str">
+      <c r="C35" s="458" t="str">
         <f>Es.1!L13</f>
         <v xml:space="preserve">Ricerca - lista vuota - annulla </v>
       </c>
-      <c r="D35" s="456"/>
-      <c r="E35" s="457" t="s">
+      <c r="D35" s="459"/>
+      <c r="E35" s="460" t="s">
         <v>498</v>
       </c>
-      <c r="F35" s="456"/>
+      <c r="F35" s="459"/>
       <c r="G35" s="189"/>
       <c r="H35" s="131"/>
       <c r="I35" s="190"/>
@@ -11321,15 +11321,15 @@
       <c r="B36" s="188" t="s">
         <v>75</v>
       </c>
-      <c r="C36" s="455" t="str">
+      <c r="C36" s="458" t="str">
         <f>Es.1!L14</f>
         <v>Checklist Accessibilità</v>
       </c>
-      <c r="D36" s="456"/>
-      <c r="E36" s="457" t="s">
+      <c r="D36" s="459"/>
+      <c r="E36" s="460" t="s">
         <v>498</v>
       </c>
-      <c r="F36" s="456"/>
+      <c r="F36" s="459"/>
       <c r="G36" s="189"/>
       <c r="H36" s="131"/>
       <c r="I36" s="190"/>
@@ -11342,15 +11342,15 @@
       <c r="B37" s="188" t="s">
         <v>75</v>
       </c>
-      <c r="C37" s="455" t="str">
+      <c r="C37" s="458" t="str">
         <f>Es.1!L15</f>
         <v>Performance Test su ricerca dati progetto</v>
       </c>
-      <c r="D37" s="456"/>
-      <c r="E37" s="457" t="s">
+      <c r="D37" s="459"/>
+      <c r="E37" s="460" t="s">
         <v>498</v>
       </c>
-      <c r="F37" s="456"/>
+      <c r="F37" s="459"/>
       <c r="G37" s="189"/>
       <c r="H37" s="131"/>
       <c r="I37" s="190"/>
@@ -11362,14 +11362,14 @@
       <c r="B38" s="215" t="s">
         <v>81</v>
       </c>
-      <c r="C38" s="460" t="s">
+      <c r="C38" s="455" t="s">
         <v>82</v>
       </c>
-      <c r="D38" s="461"/>
-      <c r="E38" s="479" t="s">
+      <c r="D38" s="456"/>
+      <c r="E38" s="457" t="s">
         <v>83</v>
       </c>
-      <c r="F38" s="461"/>
+      <c r="F38" s="456"/>
       <c r="G38" s="211">
         <v>1</v>
       </c>
@@ -11565,6 +11565,24 @@
     </row>
   </sheetData>
   <mergeCells count="32">
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="E28:F28"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="D1:I1"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="D2:I2"/>
     <mergeCell ref="C38:D38"/>
     <mergeCell ref="E38:F38"/>
     <mergeCell ref="C33:D33"/>
@@ -11579,24 +11597,6 @@
     <mergeCell ref="E35:F35"/>
     <mergeCell ref="C36:D36"/>
     <mergeCell ref="E36:F36"/>
-    <mergeCell ref="D1:I1"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="E3:F3"/>
-    <mergeCell ref="D2:I2"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="E30:F30"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="E28:F28"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="E13:F13"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.28999999999999998" right="0.55000000000000004" top="0.43" bottom="0.4" header="0.23" footer="0.23"/>
@@ -11614,18 +11614,18 @@
   <controls>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="453634" r:id="rId4" name="Btn_InsLayout">
+        <control shapeId="453636" r:id="rId4" name="Btn_Duplicate">
           <controlPr defaultSize="0" autoLine="0" autoPict="0" r:id="rId5">
             <anchor moveWithCells="1">
               <from>
-                <xdr:col>3</xdr:col>
-                <xdr:colOff>9525</xdr:colOff>
+                <xdr:col>4</xdr:col>
+                <xdr:colOff>561975</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>19050</xdr:rowOff>
               </from>
               <to>
-                <xdr:col>3</xdr:col>
-                <xdr:colOff>1676400</xdr:colOff>
+                <xdr:col>4</xdr:col>
+                <xdr:colOff>1905000</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>371475</xdr:rowOff>
               </to>
@@ -11634,7 +11634,7 @@
         </control>
       </mc:Choice>
       <mc:Fallback>
-        <control shapeId="453634" r:id="rId4" name="Btn_InsLayout"/>
+        <control shapeId="453636" r:id="rId4" name="Btn_Duplicate"/>
       </mc:Fallback>
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -11664,18 +11664,18 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="453636" r:id="rId8" name="Btn_Duplicate">
+        <control shapeId="453634" r:id="rId8" name="Btn_InsLayout">
           <controlPr defaultSize="0" autoLine="0" autoPict="0" r:id="rId9">
             <anchor moveWithCells="1">
               <from>
-                <xdr:col>4</xdr:col>
-                <xdr:colOff>561975</xdr:colOff>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>9525</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>19050</xdr:rowOff>
               </from>
               <to>
-                <xdr:col>4</xdr:col>
-                <xdr:colOff>1905000</xdr:colOff>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>1676400</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>371475</xdr:rowOff>
               </to>
@@ -11684,7 +11684,7 @@
         </control>
       </mc:Choice>
       <mc:Fallback>
-        <control shapeId="453636" r:id="rId8" name="Btn_Duplicate"/>
+        <control shapeId="453634" r:id="rId8" name="Btn_InsLayout"/>
       </mc:Fallback>
     </mc:AlternateContent>
   </controls>
@@ -11707,10 +11707,10 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18.75" customHeight="1">
       <c r="A1" s="2"/>
-      <c r="B1" s="506"/>
-      <c r="C1" s="506"/>
-      <c r="D1" s="506"/>
-      <c r="E1" s="507"/>
+      <c r="B1" s="499"/>
+      <c r="C1" s="499"/>
+      <c r="D1" s="499"/>
+      <c r="E1" s="500"/>
       <c r="F1" s="4"/>
       <c r="G1" s="22"/>
       <c r="H1" s="22"/>
@@ -11736,13 +11736,13 @@
       <c r="AB1" s="22"/>
     </row>
     <row r="2" spans="1:28" ht="30.75" customHeight="1">
-      <c r="A2" s="508" t="s">
+      <c r="A2" s="501" t="s">
         <v>43</v>
       </c>
-      <c r="B2" s="509"/>
-      <c r="C2" s="509"/>
-      <c r="D2" s="509"/>
-      <c r="E2" s="509"/>
+      <c r="B2" s="502"/>
+      <c r="C2" s="502"/>
+      <c r="D2" s="502"/>
+      <c r="E2" s="502"/>
       <c r="F2" s="88"/>
       <c r="G2" s="22"/>
       <c r="H2" s="22"/>
@@ -11771,12 +11771,12 @@
       <c r="A3" s="86" t="s">
         <v>541</v>
       </c>
-      <c r="B3" s="510" t="s">
+      <c r="B3" s="503" t="s">
         <v>286</v>
       </c>
-      <c r="C3" s="511"/>
-      <c r="D3" s="511"/>
-      <c r="E3" s="511"/>
+      <c r="C3" s="504"/>
+      <c r="D3" s="504"/>
+      <c r="E3" s="504"/>
       <c r="F3" s="4"/>
       <c r="G3" s="22"/>
       <c r="H3" s="22"/>
@@ -11803,11 +11803,11 @@
     </row>
     <row r="4" spans="1:28" ht="12.75" hidden="1" customHeight="1">
       <c r="A4" s="31"/>
-      <c r="B4" s="497" t="s">
+      <c r="B4" s="496" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="498"/>
-      <c r="D4" s="498"/>
+      <c r="C4" s="497"/>
+      <c r="D4" s="497"/>
       <c r="E4" s="5"/>
       <c r="F4" s="4"/>
       <c r="G4" s="22"/>
@@ -11835,9 +11835,9 @@
     </row>
     <row r="5" spans="1:28" ht="12.75" hidden="1" customHeight="1">
       <c r="A5" s="31"/>
-      <c r="B5" s="497"/>
-      <c r="C5" s="498"/>
-      <c r="D5" s="498"/>
+      <c r="B5" s="496"/>
+      <c r="C5" s="497"/>
+      <c r="D5" s="497"/>
       <c r="E5" s="5"/>
       <c r="F5" s="4"/>
       <c r="G5" s="22"/>
@@ -11865,9 +11865,9 @@
     </row>
     <row r="6" spans="1:28" ht="12.75" hidden="1" customHeight="1">
       <c r="A6" s="31"/>
-      <c r="B6" s="497"/>
-      <c r="C6" s="498"/>
-      <c r="D6" s="498"/>
+      <c r="B6" s="496"/>
+      <c r="C6" s="497"/>
+      <c r="D6" s="497"/>
       <c r="E6" s="5"/>
       <c r="F6" s="4"/>
       <c r="G6" s="22"/>
@@ -11897,11 +11897,11 @@
       <c r="A7" s="31" t="s">
         <v>279</v>
       </c>
-      <c r="B7" s="497" t="s">
+      <c r="B7" s="496" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="498"/>
-      <c r="D7" s="498"/>
+      <c r="C7" s="497"/>
+      <c r="D7" s="497"/>
       <c r="E7" s="6"/>
       <c r="F7" s="4"/>
       <c r="G7" s="22"/>
@@ -11931,11 +11931,11 @@
       <c r="A8" s="31" t="s">
         <v>280</v>
       </c>
-      <c r="B8" s="497">
+      <c r="B8" s="496">
         <v>1</v>
       </c>
-      <c r="C8" s="498"/>
-      <c r="D8" s="498"/>
+      <c r="C8" s="497"/>
+      <c r="D8" s="497"/>
       <c r="E8" s="6"/>
       <c r="F8" s="4"/>
       <c r="G8" s="22"/>
@@ -11965,11 +11965,11 @@
       <c r="A9" s="31" t="s">
         <v>288</v>
       </c>
-      <c r="B9" s="497" t="s">
+      <c r="B9" s="496" t="s">
         <v>362</v>
       </c>
-      <c r="C9" s="498"/>
-      <c r="D9" s="498"/>
+      <c r="C9" s="497"/>
+      <c r="D9" s="497"/>
       <c r="E9" s="6"/>
       <c r="F9" s="4"/>
       <c r="G9" s="22"/>
@@ -11999,11 +11999,11 @@
       <c r="A10" s="31" t="s">
         <v>228</v>
       </c>
-      <c r="B10" s="497" t="s">
+      <c r="B10" s="496" t="s">
         <v>289</v>
       </c>
-      <c r="C10" s="498"/>
-      <c r="D10" s="498"/>
+      <c r="C10" s="497"/>
+      <c r="D10" s="497"/>
       <c r="E10" s="6"/>
       <c r="F10" s="4"/>
       <c r="G10" s="22"/>
@@ -12033,11 +12033,11 @@
       <c r="A11" s="31" t="s">
         <v>251</v>
       </c>
-      <c r="B11" s="497">
+      <c r="B11" s="496">
         <v>10</v>
       </c>
-      <c r="C11" s="498"/>
-      <c r="D11" s="498"/>
+      <c r="C11" s="497"/>
+      <c r="D11" s="497"/>
       <c r="E11" s="5" t="s">
         <v>290</v>
       </c>
@@ -12067,9 +12067,9 @@
     </row>
     <row r="12" spans="1:28" ht="18" hidden="1" customHeight="1">
       <c r="A12" s="31"/>
-      <c r="B12" s="497"/>
-      <c r="C12" s="498"/>
-      <c r="D12" s="498"/>
+      <c r="B12" s="496"/>
+      <c r="C12" s="497"/>
+      <c r="D12" s="497"/>
       <c r="E12" s="5"/>
       <c r="F12" s="4"/>
       <c r="G12" s="22"/>
@@ -12099,11 +12099,11 @@
       <c r="A13" s="31" t="s">
         <v>291</v>
       </c>
-      <c r="B13" s="497">
+      <c r="B13" s="496">
         <v>4</v>
       </c>
-      <c r="C13" s="498"/>
-      <c r="D13" s="498"/>
+      <c r="C13" s="497"/>
+      <c r="D13" s="497"/>
       <c r="E13" s="5"/>
       <c r="F13" s="4"/>
       <c r="G13" s="22"/>
@@ -12133,11 +12133,11 @@
       <c r="A14" s="31" t="s">
         <v>292</v>
       </c>
-      <c r="B14" s="497">
+      <c r="B14" s="496">
         <v>4</v>
       </c>
-      <c r="C14" s="498"/>
-      <c r="D14" s="498"/>
+      <c r="C14" s="497"/>
+      <c r="D14" s="497"/>
       <c r="E14" s="5"/>
       <c r="F14" s="4"/>
       <c r="G14" s="22"/>
@@ -12167,9 +12167,9 @@
       <c r="A15" s="31" t="s">
         <v>363</v>
       </c>
-      <c r="B15" s="513"/>
-      <c r="C15" s="498"/>
-      <c r="D15" s="498"/>
+      <c r="B15" s="498"/>
+      <c r="C15" s="497"/>
+      <c r="D15" s="497"/>
       <c r="E15" s="5"/>
       <c r="F15" s="4"/>
       <c r="G15" s="22"/>
@@ -12196,11 +12196,11 @@
       <c r="AB15" s="22"/>
     </row>
     <row r="16" spans="1:28" ht="3.75" customHeight="1">
-      <c r="A16" s="512"/>
-      <c r="B16" s="512"/>
-      <c r="C16" s="512"/>
-      <c r="D16" s="512"/>
-      <c r="E16" s="512"/>
+      <c r="A16" s="495"/>
+      <c r="B16" s="495"/>
+      <c r="C16" s="495"/>
+      <c r="D16" s="495"/>
+      <c r="E16" s="495"/>
       <c r="F16" s="4"/>
       <c r="G16" s="22"/>
       <c r="H16" s="22"/>
@@ -12288,11 +12288,11 @@
       <c r="AB18" s="22"/>
     </row>
     <row r="19" spans="1:28" ht="12.75" customHeight="1">
-      <c r="A19" s="500" t="s">
+      <c r="A19" s="508" t="s">
         <v>294</v>
       </c>
-      <c r="B19" s="501"/>
-      <c r="C19" s="501"/>
+      <c r="B19" s="509"/>
+      <c r="C19" s="509"/>
       <c r="D19" s="490"/>
       <c r="E19" s="490"/>
       <c r="F19" s="4"/>
@@ -12323,11 +12323,11 @@
       <c r="A20" s="25" t="s">
         <v>295</v>
       </c>
-      <c r="B20" s="492">
+      <c r="B20" s="505">
         <v>4</v>
       </c>
-      <c r="C20" s="493"/>
-      <c r="D20" s="493"/>
+      <c r="C20" s="506"/>
+      <c r="D20" s="506"/>
       <c r="E20" s="7"/>
       <c r="F20" s="4"/>
       <c r="G20" s="22"/>
@@ -12357,11 +12357,11 @@
       <c r="A21" s="25" t="s">
         <v>296</v>
       </c>
-      <c r="B21" s="499">
+      <c r="B21" s="507">
         <v>0</v>
       </c>
-      <c r="C21" s="493"/>
-      <c r="D21" s="493"/>
+      <c r="C21" s="506"/>
+      <c r="D21" s="506"/>
       <c r="E21" s="7"/>
       <c r="F21" s="4"/>
       <c r="G21" s="22"/>
@@ -12391,11 +12391,11 @@
       <c r="A22" s="28" t="s">
         <v>297</v>
       </c>
-      <c r="B22" s="502">
+      <c r="B22" s="510">
         <v>1</v>
       </c>
-      <c r="C22" s="503"/>
-      <c r="D22" s="503"/>
+      <c r="C22" s="511"/>
+      <c r="D22" s="511"/>
       <c r="E22" s="7"/>
       <c r="F22" s="4"/>
       <c r="G22" s="22"/>
@@ -12425,11 +12425,11 @@
       <c r="A23" s="8" t="s">
         <v>298</v>
       </c>
-      <c r="B23" s="504" t="s">
+      <c r="B23" s="512" t="s">
         <v>540</v>
       </c>
-      <c r="C23" s="505"/>
-      <c r="D23" s="505"/>
+      <c r="C23" s="513"/>
+      <c r="D23" s="513"/>
       <c r="E23" s="9"/>
       <c r="F23" s="4"/>
       <c r="G23" s="22"/>
@@ -12456,11 +12456,11 @@
       <c r="AB23" s="22"/>
     </row>
     <row r="24" spans="1:28" ht="6.75" customHeight="1">
-      <c r="A24" s="514"/>
-      <c r="B24" s="514"/>
-      <c r="C24" s="514"/>
-      <c r="D24" s="515"/>
-      <c r="E24" s="516"/>
+      <c r="A24" s="483"/>
+      <c r="B24" s="483"/>
+      <c r="C24" s="483"/>
+      <c r="D24" s="484"/>
+      <c r="E24" s="485"/>
       <c r="F24" s="4"/>
       <c r="G24" s="22"/>
       <c r="H24" s="22"/>
@@ -12486,13 +12486,13 @@
       <c r="AB24" s="22"/>
     </row>
     <row r="25" spans="1:28" ht="12.75" customHeight="1">
-      <c r="A25" s="494" t="s">
+      <c r="A25" s="480" t="s">
         <v>405</v>
       </c>
-      <c r="B25" s="495"/>
-      <c r="C25" s="495"/>
-      <c r="D25" s="496"/>
-      <c r="E25" s="496"/>
+      <c r="B25" s="481"/>
+      <c r="C25" s="481"/>
+      <c r="D25" s="482"/>
+      <c r="E25" s="482"/>
       <c r="F25" s="4"/>
       <c r="G25" s="22"/>
       <c r="H25" s="22"/>
@@ -12748,11 +12748,11 @@
       <c r="AB31" s="22"/>
     </row>
     <row r="32" spans="1:28" ht="6.75" customHeight="1">
-      <c r="A32" s="520"/>
-      <c r="B32" s="520"/>
-      <c r="C32" s="520"/>
-      <c r="D32" s="512"/>
-      <c r="E32" s="512"/>
+      <c r="A32" s="494"/>
+      <c r="B32" s="494"/>
+      <c r="C32" s="494"/>
+      <c r="D32" s="495"/>
+      <c r="E32" s="495"/>
       <c r="F32" s="4"/>
       <c r="G32" s="22"/>
       <c r="H32" s="22"/>
@@ -12778,13 +12778,13 @@
       <c r="AB32" s="22"/>
     </row>
     <row r="33" spans="1:28" ht="12.75" customHeight="1">
-      <c r="A33" s="494" t="s">
+      <c r="A33" s="480" t="s">
         <v>406</v>
       </c>
-      <c r="B33" s="495"/>
-      <c r="C33" s="495"/>
-      <c r="D33" s="496"/>
-      <c r="E33" s="496"/>
+      <c r="B33" s="481"/>
+      <c r="C33" s="481"/>
+      <c r="D33" s="482"/>
+      <c r="E33" s="482"/>
       <c r="F33" s="4"/>
       <c r="G33" s="22"/>
       <c r="H33" s="22"/>
@@ -13040,11 +13040,11 @@
       <c r="AB39" s="22"/>
     </row>
     <row r="40" spans="1:28" ht="6.75" customHeight="1">
-      <c r="A40" s="514"/>
-      <c r="B40" s="514"/>
-      <c r="C40" s="514"/>
-      <c r="D40" s="515"/>
-      <c r="E40" s="516"/>
+      <c r="A40" s="483"/>
+      <c r="B40" s="483"/>
+      <c r="C40" s="483"/>
+      <c r="D40" s="484"/>
+      <c r="E40" s="485"/>
       <c r="F40" s="4"/>
       <c r="G40" s="22"/>
       <c r="H40" s="22"/>
@@ -13070,13 +13070,13 @@
       <c r="AB40" s="22"/>
     </row>
     <row r="41" spans="1:28" ht="12.75" customHeight="1">
-      <c r="A41" s="494" t="s">
+      <c r="A41" s="480" t="s">
         <v>407</v>
       </c>
-      <c r="B41" s="495"/>
-      <c r="C41" s="495"/>
-      <c r="D41" s="496"/>
-      <c r="E41" s="496"/>
+      <c r="B41" s="481"/>
+      <c r="C41" s="481"/>
+      <c r="D41" s="482"/>
+      <c r="E41" s="482"/>
       <c r="F41" s="4"/>
       <c r="G41" s="22"/>
       <c r="H41" s="22"/>
@@ -13338,11 +13338,11 @@
       <c r="AB47" s="22"/>
     </row>
     <row r="48" spans="1:28" ht="6.75" customHeight="1">
-      <c r="A48" s="514"/>
-      <c r="B48" s="514"/>
-      <c r="C48" s="514"/>
-      <c r="D48" s="515"/>
-      <c r="E48" s="516"/>
+      <c r="A48" s="483"/>
+      <c r="B48" s="483"/>
+      <c r="C48" s="483"/>
+      <c r="D48" s="484"/>
+      <c r="E48" s="485"/>
       <c r="F48" s="4"/>
       <c r="G48" s="22"/>
       <c r="H48" s="22"/>
@@ -13368,13 +13368,13 @@
       <c r="AB48" s="22"/>
     </row>
     <row r="49" spans="1:28" ht="12.75" customHeight="1">
-      <c r="A49" s="494" t="s">
+      <c r="A49" s="480" t="s">
         <v>285</v>
       </c>
-      <c r="B49" s="495"/>
-      <c r="C49" s="495"/>
-      <c r="D49" s="496"/>
-      <c r="E49" s="496"/>
+      <c r="B49" s="481"/>
+      <c r="C49" s="481"/>
+      <c r="D49" s="482"/>
+      <c r="E49" s="482"/>
       <c r="F49" s="4"/>
       <c r="G49" s="22"/>
       <c r="H49" s="22"/>
@@ -13630,11 +13630,11 @@
       <c r="AB55" s="22"/>
     </row>
     <row r="56" spans="1:28" ht="3" customHeight="1">
-      <c r="A56" s="512"/>
-      <c r="B56" s="512"/>
-      <c r="C56" s="512"/>
-      <c r="D56" s="512"/>
-      <c r="E56" s="512"/>
+      <c r="A56" s="495"/>
+      <c r="B56" s="495"/>
+      <c r="C56" s="495"/>
+      <c r="D56" s="495"/>
+      <c r="E56" s="495"/>
       <c r="F56" s="4"/>
       <c r="G56" s="22"/>
       <c r="H56" s="22"/>
@@ -13758,11 +13758,11 @@
       <c r="B60" s="21" t="s">
         <v>300</v>
       </c>
-      <c r="C60" s="517" t="s">
+      <c r="C60" s="491" t="s">
         <v>301</v>
       </c>
-      <c r="D60" s="518"/>
-      <c r="E60" s="519"/>
+      <c r="D60" s="492"/>
+      <c r="E60" s="493"/>
       <c r="F60" s="4"/>
       <c r="G60" s="22"/>
       <c r="H60" s="22"/>
@@ -13794,11 +13794,11 @@
       <c r="B61" s="30" t="s">
         <v>152</v>
       </c>
-      <c r="C61" s="483" t="s">
+      <c r="C61" s="486" t="s">
         <v>258</v>
       </c>
-      <c r="D61" s="484"/>
-      <c r="E61" s="491"/>
+      <c r="D61" s="487"/>
+      <c r="E61" s="488"/>
       <c r="F61" s="4"/>
       <c r="G61" s="22"/>
       <c r="H61" s="22"/>
@@ -13830,11 +13830,11 @@
       <c r="B62" s="30" t="s">
         <v>153</v>
       </c>
-      <c r="C62" s="483" t="s">
+      <c r="C62" s="486" t="s">
         <v>258</v>
       </c>
-      <c r="D62" s="484"/>
-      <c r="E62" s="491"/>
+      <c r="D62" s="487"/>
+      <c r="E62" s="488"/>
       <c r="F62" s="4"/>
       <c r="G62" s="22"/>
       <c r="H62" s="22"/>
@@ -13866,11 +13866,11 @@
       <c r="B63" s="30" t="s">
         <v>154</v>
       </c>
-      <c r="C63" s="483" t="s">
+      <c r="C63" s="486" t="s">
         <v>258</v>
       </c>
-      <c r="D63" s="484"/>
-      <c r="E63" s="491"/>
+      <c r="D63" s="487"/>
+      <c r="E63" s="488"/>
       <c r="F63" s="4"/>
       <c r="G63" s="22"/>
       <c r="H63" s="22"/>
@@ -13902,11 +13902,11 @@
       <c r="B64" s="30" t="s">
         <v>141</v>
       </c>
-      <c r="C64" s="483" t="s">
+      <c r="C64" s="486" t="s">
         <v>258</v>
       </c>
-      <c r="D64" s="484"/>
-      <c r="E64" s="491"/>
+      <c r="D64" s="487"/>
+      <c r="E64" s="488"/>
       <c r="F64" s="4"/>
       <c r="G64" s="22"/>
       <c r="H64" s="22"/>
@@ -13938,11 +13938,11 @@
       <c r="B65" s="30" t="s">
         <v>155</v>
       </c>
-      <c r="C65" s="483" t="s">
+      <c r="C65" s="486" t="s">
         <v>258</v>
       </c>
-      <c r="D65" s="484"/>
-      <c r="E65" s="491"/>
+      <c r="D65" s="487"/>
+      <c r="E65" s="488"/>
       <c r="F65" s="4"/>
       <c r="G65" s="22"/>
       <c r="H65" s="22"/>
@@ -13974,11 +13974,11 @@
       <c r="B66" s="30" t="s">
         <v>144</v>
       </c>
-      <c r="C66" s="483" t="s">
+      <c r="C66" s="486" t="s">
         <v>258</v>
       </c>
-      <c r="D66" s="484"/>
-      <c r="E66" s="491"/>
+      <c r="D66" s="487"/>
+      <c r="E66" s="488"/>
       <c r="F66" s="4"/>
       <c r="G66" s="22"/>
       <c r="H66" s="22"/>
@@ -14010,11 +14010,11 @@
       <c r="B67" s="30" t="s">
         <v>156</v>
       </c>
-      <c r="C67" s="483" t="s">
+      <c r="C67" s="486" t="s">
         <v>258</v>
       </c>
-      <c r="D67" s="484"/>
-      <c r="E67" s="491"/>
+      <c r="D67" s="487"/>
+      <c r="E67" s="488"/>
       <c r="F67" s="4"/>
       <c r="G67" s="22"/>
       <c r="H67" s="22"/>
@@ -14046,11 +14046,11 @@
       <c r="B68" s="30" t="s">
         <v>145</v>
       </c>
-      <c r="C68" s="483" t="s">
+      <c r="C68" s="486" t="s">
         <v>258</v>
       </c>
-      <c r="D68" s="484"/>
-      <c r="E68" s="491"/>
+      <c r="D68" s="487"/>
+      <c r="E68" s="488"/>
       <c r="F68" s="4"/>
       <c r="G68" s="22"/>
       <c r="H68" s="22"/>
@@ -14082,11 +14082,11 @@
       <c r="B69" s="30" t="s">
         <v>146</v>
       </c>
-      <c r="C69" s="483" t="s">
+      <c r="C69" s="486" t="s">
         <v>258</v>
       </c>
-      <c r="D69" s="484"/>
-      <c r="E69" s="491"/>
+      <c r="D69" s="487"/>
+      <c r="E69" s="488"/>
       <c r="F69" s="4"/>
       <c r="G69" s="22"/>
       <c r="H69" s="22"/>
@@ -14118,11 +14118,11 @@
       <c r="B70" s="30" t="s">
         <v>148</v>
       </c>
-      <c r="C70" s="483" t="s">
+      <c r="C70" s="486" t="s">
         <v>258</v>
       </c>
-      <c r="D70" s="484"/>
-      <c r="E70" s="491"/>
+      <c r="D70" s="487"/>
+      <c r="E70" s="488"/>
       <c r="F70" s="4"/>
       <c r="G70" s="22"/>
       <c r="H70" s="22"/>
@@ -14154,11 +14154,11 @@
       <c r="B71" s="30" t="s">
         <v>159</v>
       </c>
-      <c r="C71" s="483" t="s">
+      <c r="C71" s="486" t="s">
         <v>258</v>
       </c>
-      <c r="D71" s="484"/>
-      <c r="E71" s="491"/>
+      <c r="D71" s="487"/>
+      <c r="E71" s="488"/>
       <c r="F71" s="4"/>
       <c r="G71" s="22"/>
       <c r="H71" s="22"/>
@@ -14190,11 +14190,11 @@
       <c r="B72" s="30" t="s">
         <v>162</v>
       </c>
-      <c r="C72" s="483" t="s">
+      <c r="C72" s="486" t="s">
         <v>258</v>
       </c>
-      <c r="D72" s="484"/>
-      <c r="E72" s="491"/>
+      <c r="D72" s="487"/>
+      <c r="E72" s="488"/>
       <c r="F72" s="4"/>
       <c r="G72" s="22"/>
       <c r="H72" s="22"/>
@@ -14226,11 +14226,11 @@
       <c r="B73" s="30" t="s">
         <v>164</v>
       </c>
-      <c r="C73" s="483" t="s">
+      <c r="C73" s="486" t="s">
         <v>258</v>
       </c>
-      <c r="D73" s="484"/>
-      <c r="E73" s="491"/>
+      <c r="D73" s="487"/>
+      <c r="E73" s="488"/>
       <c r="F73" s="4"/>
       <c r="G73" s="22"/>
       <c r="H73" s="22"/>
@@ -14262,13 +14262,13 @@
       <c r="B74" s="30" t="s">
         <v>163</v>
       </c>
-      <c r="C74" s="483" t="s">
+      <c r="C74" s="486" t="s">
         <v>258</v>
       </c>
-      <c r="D74" s="484" t="s">
+      <c r="D74" s="487" t="s">
         <v>258</v>
       </c>
-      <c r="E74" s="491"/>
+      <c r="E74" s="488"/>
       <c r="F74" s="4"/>
       <c r="G74" s="22"/>
       <c r="H74" s="22"/>
@@ -14300,11 +14300,11 @@
       <c r="B75" s="30" t="s">
         <v>259</v>
       </c>
-      <c r="C75" s="483" t="s">
+      <c r="C75" s="486" t="s">
         <v>258</v>
       </c>
-      <c r="D75" s="484"/>
-      <c r="E75" s="491"/>
+      <c r="D75" s="487"/>
+      <c r="E75" s="488"/>
       <c r="F75" s="4"/>
       <c r="G75" s="22"/>
       <c r="H75" s="22"/>
@@ -14336,11 +14336,11 @@
       <c r="B76" s="30" t="s">
         <v>160</v>
       </c>
-      <c r="C76" s="483" t="s">
+      <c r="C76" s="486" t="s">
         <v>258</v>
       </c>
-      <c r="D76" s="484"/>
-      <c r="E76" s="491"/>
+      <c r="D76" s="487"/>
+      <c r="E76" s="488"/>
       <c r="F76" s="4"/>
       <c r="G76" s="22"/>
       <c r="H76" s="22"/>
@@ -14372,11 +14372,11 @@
       <c r="B77" s="30" t="s">
         <v>166</v>
       </c>
-      <c r="C77" s="483" t="s">
+      <c r="C77" s="486" t="s">
         <v>258</v>
       </c>
-      <c r="D77" s="484"/>
-      <c r="E77" s="491"/>
+      <c r="D77" s="487"/>
+      <c r="E77" s="488"/>
       <c r="F77" s="4"/>
       <c r="G77" s="22"/>
       <c r="H77" s="22"/>
@@ -14408,11 +14408,11 @@
       <c r="B78" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="C78" s="483" t="s">
+      <c r="C78" s="486" t="s">
         <v>258</v>
       </c>
-      <c r="D78" s="484"/>
-      <c r="E78" s="491"/>
+      <c r="D78" s="487"/>
+      <c r="E78" s="488"/>
       <c r="F78" s="4"/>
       <c r="G78" s="22"/>
       <c r="H78" s="22"/>
@@ -14444,11 +14444,11 @@
       <c r="B79" s="30" t="s">
         <v>456</v>
       </c>
-      <c r="C79" s="483" t="s">
+      <c r="C79" s="486" t="s">
         <v>258</v>
       </c>
-      <c r="D79" s="484"/>
-      <c r="E79" s="491"/>
+      <c r="D79" s="487"/>
+      <c r="E79" s="488"/>
       <c r="F79" s="4"/>
       <c r="G79" s="22"/>
       <c r="H79" s="22"/>
@@ -14480,11 +14480,11 @@
       <c r="B80" s="30" t="s">
         <v>535</v>
       </c>
-      <c r="C80" s="483" t="s">
+      <c r="C80" s="486" t="s">
         <v>258</v>
       </c>
-      <c r="D80" s="484"/>
-      <c r="E80" s="491"/>
+      <c r="D80" s="487"/>
+      <c r="E80" s="488"/>
       <c r="F80" s="4"/>
       <c r="G80" s="22"/>
       <c r="H80" s="22"/>
@@ -14516,11 +14516,11 @@
       <c r="B81" s="143" t="s">
         <v>364</v>
       </c>
-      <c r="C81" s="483" t="s">
+      <c r="C81" s="486" t="s">
         <v>365</v>
       </c>
-      <c r="D81" s="484"/>
-      <c r="E81" s="491"/>
+      <c r="D81" s="487"/>
+      <c r="E81" s="488"/>
       <c r="G81" s="22"/>
       <c r="H81" s="22"/>
       <c r="I81" s="22"/>
@@ -14547,9 +14547,9 @@
     <row r="82" spans="1:28" ht="12.75" hidden="1" customHeight="1">
       <c r="A82" s="29"/>
       <c r="B82" s="30"/>
-      <c r="C82" s="483"/>
-      <c r="D82" s="484"/>
-      <c r="E82" s="491"/>
+      <c r="C82" s="486"/>
+      <c r="D82" s="487"/>
+      <c r="E82" s="488"/>
       <c r="G82" s="22"/>
       <c r="H82" s="22"/>
       <c r="I82" s="22"/>
@@ -14576,9 +14576,9 @@
     <row r="83" spans="1:28" ht="12.75" hidden="1" customHeight="1">
       <c r="A83" s="29"/>
       <c r="B83" s="30"/>
-      <c r="C83" s="483"/>
-      <c r="D83" s="484"/>
-      <c r="E83" s="491"/>
+      <c r="C83" s="486"/>
+      <c r="D83" s="487"/>
+      <c r="E83" s="488"/>
       <c r="G83" s="22"/>
       <c r="H83" s="22"/>
       <c r="I83" s="22"/>
@@ -14605,9 +14605,9 @@
     <row r="84" spans="1:28" ht="12.75" hidden="1" customHeight="1">
       <c r="A84" s="29"/>
       <c r="B84" s="30"/>
-      <c r="C84" s="483"/>
-      <c r="D84" s="484"/>
-      <c r="E84" s="491"/>
+      <c r="C84" s="486"/>
+      <c r="D84" s="487"/>
+      <c r="E84" s="488"/>
       <c r="G84" s="22"/>
       <c r="H84" s="22"/>
       <c r="I84" s="22"/>
@@ -14638,11 +14638,11 @@
       <c r="B85" s="30" t="s">
         <v>170</v>
       </c>
-      <c r="C85" s="483" t="s">
+      <c r="C85" s="486" t="s">
         <v>169</v>
       </c>
-      <c r="D85" s="484"/>
-      <c r="E85" s="491"/>
+      <c r="D85" s="487"/>
+      <c r="E85" s="488"/>
       <c r="G85" s="22"/>
       <c r="H85" s="22"/>
       <c r="I85" s="22"/>
@@ -14673,11 +14673,11 @@
       <c r="B86" s="30" t="s">
         <v>171</v>
       </c>
-      <c r="C86" s="483" t="s">
+      <c r="C86" s="486" t="s">
         <v>169</v>
       </c>
-      <c r="D86" s="484"/>
-      <c r="E86" s="491"/>
+      <c r="D86" s="487"/>
+      <c r="E86" s="488"/>
       <c r="G86" s="22"/>
       <c r="H86" s="22"/>
       <c r="I86" s="22"/>
@@ -14708,11 +14708,11 @@
       <c r="B87" s="30" t="s">
         <v>172</v>
       </c>
-      <c r="C87" s="483" t="s">
+      <c r="C87" s="486" t="s">
         <v>169</v>
       </c>
-      <c r="D87" s="484"/>
-      <c r="E87" s="491"/>
+      <c r="D87" s="487"/>
+      <c r="E87" s="488"/>
       <c r="G87" s="22"/>
       <c r="H87" s="22"/>
       <c r="I87" s="22"/>
@@ -14743,11 +14743,11 @@
       <c r="B88" s="30" t="s">
         <v>173</v>
       </c>
-      <c r="C88" s="483" t="s">
+      <c r="C88" s="486" t="s">
         <v>169</v>
       </c>
-      <c r="D88" s="484"/>
-      <c r="E88" s="491"/>
+      <c r="D88" s="487"/>
+      <c r="E88" s="488"/>
       <c r="G88" s="22"/>
       <c r="H88" s="22"/>
       <c r="I88" s="22"/>
@@ -14778,11 +14778,11 @@
       <c r="B89" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="C89" s="483" t="s">
+      <c r="C89" s="486" t="s">
         <v>169</v>
       </c>
-      <c r="D89" s="484"/>
-      <c r="E89" s="491"/>
+      <c r="D89" s="487"/>
+      <c r="E89" s="488"/>
       <c r="G89" s="22"/>
       <c r="H89" s="22"/>
       <c r="I89" s="22"/>
@@ -14963,22 +14963,22 @@
       <c r="B95" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="C95" s="483" t="s">
+      <c r="C95" s="486" t="s">
         <v>183</v>
       </c>
-      <c r="D95" s="484"/>
-      <c r="E95" s="484"/>
+      <c r="D95" s="487"/>
+      <c r="E95" s="487"/>
       <c r="G95" s="22"/>
       <c r="H95" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="I95" s="480" t="s">
+      <c r="I95" s="516" t="s">
         <v>455</v>
       </c>
-      <c r="J95" s="481"/>
-      <c r="K95" s="481"/>
-      <c r="L95" s="481"/>
-      <c r="M95" s="482"/>
+      <c r="J95" s="517"/>
+      <c r="K95" s="517"/>
+      <c r="L95" s="517"/>
+      <c r="M95" s="518"/>
       <c r="N95" s="22"/>
       <c r="O95" s="22"/>
       <c r="P95" s="22"/>
@@ -15002,11 +15002,11 @@
       <c r="B96" s="33" t="s">
         <v>78</v>
       </c>
-      <c r="C96" s="483" t="s">
+      <c r="C96" s="486" t="s">
         <v>210</v>
       </c>
-      <c r="D96" s="484"/>
-      <c r="E96" s="484"/>
+      <c r="D96" s="487"/>
+      <c r="E96" s="487"/>
       <c r="G96" s="22"/>
       <c r="H96" s="133" t="s">
         <v>454</v>
@@ -15047,11 +15047,11 @@
         <v>11</v>
       </c>
       <c r="B97" s="33"/>
-      <c r="C97" s="483" t="s">
+      <c r="C97" s="486" t="s">
         <v>211</v>
       </c>
-      <c r="D97" s="484"/>
-      <c r="E97" s="484"/>
+      <c r="D97" s="487"/>
+      <c r="E97" s="487"/>
       <c r="G97" s="22"/>
       <c r="H97" s="132">
         <v>1</v>
@@ -15099,11 +15099,11 @@
       <c r="B98" s="33" t="s">
         <v>495</v>
       </c>
-      <c r="C98" s="483" t="s">
+      <c r="C98" s="486" t="s">
         <v>402</v>
       </c>
-      <c r="D98" s="484"/>
-      <c r="E98" s="484"/>
+      <c r="D98" s="487"/>
+      <c r="E98" s="487"/>
       <c r="G98" s="22"/>
       <c r="H98" s="132">
         <v>2</v>
@@ -15149,9 +15149,9 @@
         <v>96</v>
       </c>
       <c r="B99" s="33"/>
-      <c r="C99" s="483"/>
-      <c r="D99" s="484"/>
-      <c r="E99" s="484"/>
+      <c r="C99" s="486"/>
+      <c r="D99" s="487"/>
+      <c r="E99" s="487"/>
       <c r="G99" s="22"/>
       <c r="H99" s="132">
         <v>3</v>
@@ -15193,13 +15193,13 @@
       <c r="AB99" s="22"/>
     </row>
     <row r="100" spans="1:28" ht="12.75" customHeight="1">
-      <c r="A100" s="485" t="s">
+      <c r="A100" s="519" t="s">
         <v>431</v>
       </c>
-      <c r="B100" s="486"/>
-      <c r="C100" s="486"/>
-      <c r="D100" s="486"/>
-      <c r="E100" s="486"/>
+      <c r="B100" s="520"/>
+      <c r="C100" s="520"/>
+      <c r="D100" s="520"/>
+      <c r="E100" s="520"/>
       <c r="G100" s="22"/>
       <c r="H100" s="132">
         <v>4</v>
@@ -15247,11 +15247,11 @@
       <c r="B101" s="85" t="s">
         <v>152</v>
       </c>
-      <c r="C101" s="483" t="s">
+      <c r="C101" s="486" t="s">
         <v>401</v>
       </c>
-      <c r="D101" s="484"/>
-      <c r="E101" s="484"/>
+      <c r="D101" s="487"/>
+      <c r="E101" s="487"/>
       <c r="G101" s="22"/>
       <c r="H101" s="132">
         <v>5</v>
@@ -15299,11 +15299,11 @@
       <c r="B102" s="85" t="s">
         <v>153</v>
       </c>
-      <c r="C102" s="483" t="s">
+      <c r="C102" s="486" t="s">
         <v>401</v>
       </c>
-      <c r="D102" s="484"/>
-      <c r="E102" s="484"/>
+      <c r="D102" s="487"/>
+      <c r="E102" s="487"/>
       <c r="G102" s="22"/>
       <c r="H102" s="23" t="s">
         <v>451</v>
@@ -15336,11 +15336,11 @@
       <c r="B103" s="85" t="s">
         <v>154</v>
       </c>
-      <c r="C103" s="483" t="s">
+      <c r="C103" s="486" t="s">
         <v>401</v>
       </c>
-      <c r="D103" s="484"/>
-      <c r="E103" s="484"/>
+      <c r="D103" s="487"/>
+      <c r="E103" s="487"/>
       <c r="G103" s="22"/>
       <c r="H103" s="22" t="s">
         <v>452</v>
@@ -15375,11 +15375,11 @@
       <c r="B104" s="85" t="s">
         <v>155</v>
       </c>
-      <c r="C104" s="483" t="s">
+      <c r="C104" s="486" t="s">
         <v>401</v>
       </c>
-      <c r="D104" s="484"/>
-      <c r="E104" s="484"/>
+      <c r="D104" s="487"/>
+      <c r="E104" s="487"/>
       <c r="G104" s="22"/>
       <c r="H104" s="22" t="s">
         <v>66</v>
@@ -15414,11 +15414,11 @@
       <c r="B105" s="85" t="s">
         <v>156</v>
       </c>
-      <c r="C105" s="483" t="s">
+      <c r="C105" s="486" t="s">
         <v>401</v>
       </c>
-      <c r="D105" s="484"/>
-      <c r="E105" s="484"/>
+      <c r="D105" s="487"/>
+      <c r="E105" s="487"/>
       <c r="G105" s="22"/>
       <c r="H105" s="22" t="s">
         <v>439</v>
@@ -15453,11 +15453,11 @@
       <c r="B106" s="85" t="s">
         <v>145</v>
       </c>
-      <c r="C106" s="483" t="s">
+      <c r="C106" s="486" t="s">
         <v>401</v>
       </c>
-      <c r="D106" s="484"/>
-      <c r="E106" s="484"/>
+      <c r="D106" s="487"/>
+      <c r="E106" s="487"/>
       <c r="G106" s="22"/>
       <c r="H106" s="22" t="s">
         <v>441</v>
@@ -15492,11 +15492,11 @@
       <c r="B107" s="85" t="s">
         <v>146</v>
       </c>
-      <c r="C107" s="483" t="s">
+      <c r="C107" s="486" t="s">
         <v>401</v>
       </c>
-      <c r="D107" s="484"/>
-      <c r="E107" s="484"/>
+      <c r="D107" s="487"/>
+      <c r="E107" s="487"/>
       <c r="G107" s="22"/>
       <c r="H107" s="22" t="s">
         <v>443</v>
@@ -15531,11 +15531,11 @@
       <c r="B108" s="101" t="s">
         <v>46</v>
       </c>
-      <c r="C108" s="483" t="s">
+      <c r="C108" s="486" t="s">
         <v>47</v>
       </c>
-      <c r="D108" s="484"/>
-      <c r="E108" s="484"/>
+      <c r="D108" s="487"/>
+      <c r="E108" s="487"/>
       <c r="G108" s="22"/>
       <c r="H108" s="22" t="s">
         <v>445</v>
@@ -15564,13 +15564,13 @@
       <c r="AB108" s="22"/>
     </row>
     <row r="109" spans="1:28" ht="12.75" customHeight="1">
-      <c r="A109" s="485" t="s">
+      <c r="A109" s="519" t="s">
         <v>432</v>
       </c>
-      <c r="B109" s="486"/>
-      <c r="C109" s="486"/>
-      <c r="D109" s="486"/>
-      <c r="E109" s="486"/>
+      <c r="B109" s="520"/>
+      <c r="C109" s="520"/>
+      <c r="D109" s="520"/>
+      <c r="E109" s="520"/>
       <c r="G109" s="22"/>
       <c r="H109" s="138" t="s">
         <v>449</v>
@@ -15603,11 +15603,11 @@
       <c r="B110" s="85" t="s">
         <v>153</v>
       </c>
-      <c r="C110" s="483" t="s">
+      <c r="C110" s="486" t="s">
         <v>401</v>
       </c>
-      <c r="D110" s="484"/>
-      <c r="E110" s="484"/>
+      <c r="D110" s="487"/>
+      <c r="E110" s="487"/>
       <c r="G110" s="22"/>
       <c r="H110" s="22" t="s">
         <v>448</v>
@@ -15640,11 +15640,11 @@
       <c r="B111" s="85" t="s">
         <v>154</v>
       </c>
-      <c r="C111" s="483" t="s">
+      <c r="C111" s="486" t="s">
         <v>401</v>
       </c>
-      <c r="D111" s="484"/>
-      <c r="E111" s="484"/>
+      <c r="D111" s="487"/>
+      <c r="E111" s="487"/>
       <c r="G111" s="22"/>
       <c r="H111" s="22"/>
       <c r="I111" s="22"/>
@@ -15675,11 +15675,11 @@
       <c r="B112" s="85" t="s">
         <v>141</v>
       </c>
-      <c r="C112" s="483" t="s">
+      <c r="C112" s="486" t="s">
         <v>401</v>
       </c>
-      <c r="D112" s="484"/>
-      <c r="E112" s="484"/>
+      <c r="D112" s="487"/>
+      <c r="E112" s="487"/>
       <c r="G112" s="22"/>
       <c r="I112" s="22"/>
       <c r="J112" s="22"/>
@@ -15709,11 +15709,11 @@
       <c r="B113" s="85" t="s">
         <v>155</v>
       </c>
-      <c r="C113" s="483" t="s">
+      <c r="C113" s="486" t="s">
         <v>401</v>
       </c>
-      <c r="D113" s="484"/>
-      <c r="E113" s="484"/>
+      <c r="D113" s="487"/>
+      <c r="E113" s="487"/>
       <c r="G113" s="22"/>
       <c r="H113" s="22"/>
       <c r="I113" s="22"/>
@@ -15744,11 +15744,11 @@
       <c r="B114" s="85" t="s">
         <v>144</v>
       </c>
-      <c r="C114" s="483" t="s">
+      <c r="C114" s="486" t="s">
         <v>401</v>
       </c>
-      <c r="D114" s="484"/>
-      <c r="E114" s="484"/>
+      <c r="D114" s="487"/>
+      <c r="E114" s="487"/>
       <c r="G114" s="22"/>
       <c r="H114" s="22"/>
       <c r="I114" s="22"/>
@@ -15773,13 +15773,13 @@
       <c r="AB114" s="22"/>
     </row>
     <row r="115" spans="1:28" ht="12.75" customHeight="1">
-      <c r="A115" s="485" t="s">
+      <c r="A115" s="519" t="s">
         <v>397</v>
       </c>
-      <c r="B115" s="486"/>
-      <c r="C115" s="486"/>
-      <c r="D115" s="486"/>
-      <c r="E115" s="486"/>
+      <c r="B115" s="520"/>
+      <c r="C115" s="520"/>
+      <c r="D115" s="520"/>
+      <c r="E115" s="520"/>
       <c r="G115" s="22"/>
       <c r="H115" s="22"/>
       <c r="I115" s="22"/>
@@ -15810,11 +15810,11 @@
       <c r="B116" s="85">
         <v>4</v>
       </c>
-      <c r="C116" s="483" t="s">
+      <c r="C116" s="486" t="s">
         <v>399</v>
       </c>
-      <c r="D116" s="484"/>
-      <c r="E116" s="484"/>
+      <c r="D116" s="487"/>
+      <c r="E116" s="487"/>
       <c r="G116" s="22"/>
       <c r="H116" s="22"/>
       <c r="I116" s="22"/>
@@ -15845,11 +15845,11 @@
       <c r="B117" s="85">
         <v>5</v>
       </c>
-      <c r="C117" s="483" t="s">
+      <c r="C117" s="486" t="s">
         <v>399</v>
       </c>
-      <c r="D117" s="484"/>
-      <c r="E117" s="484"/>
+      <c r="D117" s="487"/>
+      <c r="E117" s="487"/>
       <c r="G117" s="22"/>
       <c r="H117" s="22"/>
       <c r="I117" s="22"/>
@@ -15878,11 +15878,11 @@
         <v>404</v>
       </c>
       <c r="B118" s="107"/>
-      <c r="C118" s="483" t="s">
+      <c r="C118" s="486" t="s">
         <v>403</v>
       </c>
-      <c r="D118" s="484"/>
-      <c r="E118" s="484"/>
+      <c r="D118" s="487"/>
+      <c r="E118" s="487"/>
       <c r="G118" s="22"/>
       <c r="H118" s="22"/>
       <c r="I118" s="22"/>
@@ -15913,11 +15913,11 @@
       <c r="B119" s="85" t="s">
         <v>90</v>
       </c>
-      <c r="C119" s="483" t="s">
+      <c r="C119" s="486" t="s">
         <v>402</v>
       </c>
-      <c r="D119" s="484"/>
-      <c r="E119" s="484"/>
+      <c r="D119" s="487"/>
+      <c r="E119" s="487"/>
       <c r="G119" s="22"/>
       <c r="H119" s="22"/>
       <c r="I119" s="22"/>
@@ -15973,9 +15973,9 @@
     <row r="121" spans="1:28" ht="12.75" hidden="1" customHeight="1">
       <c r="A121" s="34"/>
       <c r="B121" s="85"/>
-      <c r="C121" s="483"/>
-      <c r="D121" s="484"/>
-      <c r="E121" s="484"/>
+      <c r="C121" s="486"/>
+      <c r="D121" s="487"/>
+      <c r="E121" s="487"/>
       <c r="G121" s="22"/>
       <c r="H121" s="22"/>
       <c r="I121" s="22"/>
@@ -16002,11 +16002,11 @@
     <row r="122" spans="1:28" ht="12.75" hidden="1" customHeight="1">
       <c r="A122" s="208"/>
       <c r="B122" s="209"/>
-      <c r="C122" s="483" t="s">
+      <c r="C122" s="486" t="s">
         <v>382</v>
       </c>
-      <c r="D122" s="484"/>
-      <c r="E122" s="484"/>
+      <c r="D122" s="487"/>
+      <c r="E122" s="487"/>
       <c r="G122" s="22"/>
       <c r="H122" s="22"/>
       <c r="I122" s="22"/>
@@ -16097,9 +16097,9 @@
       <c r="B125" s="84" t="s">
         <v>76</v>
       </c>
-      <c r="C125" s="487"/>
-      <c r="D125" s="488"/>
-      <c r="E125" s="488"/>
+      <c r="C125" s="514"/>
+      <c r="D125" s="515"/>
+      <c r="E125" s="515"/>
       <c r="G125" s="22"/>
       <c r="H125" s="22"/>
       <c r="I125" s="22"/>
@@ -16128,9 +16128,9 @@
         <v>430</v>
       </c>
       <c r="B126" s="84"/>
-      <c r="C126" s="487"/>
-      <c r="D126" s="488"/>
-      <c r="E126" s="488"/>
+      <c r="C126" s="514"/>
+      <c r="D126" s="515"/>
+      <c r="E126" s="515"/>
       <c r="G126" s="22"/>
       <c r="H126" s="22"/>
       <c r="I126" s="22"/>
@@ -16161,9 +16161,9 @@
       <c r="B127" s="84" t="s">
         <v>77</v>
       </c>
-      <c r="C127" s="487"/>
-      <c r="D127" s="488"/>
-      <c r="E127" s="488"/>
+      <c r="C127" s="514"/>
+      <c r="D127" s="515"/>
+      <c r="E127" s="515"/>
       <c r="G127" s="22"/>
       <c r="H127" s="22"/>
       <c r="I127" s="22"/>
@@ -16194,9 +16194,9 @@
       <c r="B128" s="111" t="s">
         <v>45</v>
       </c>
-      <c r="C128" s="487"/>
-      <c r="D128" s="488"/>
-      <c r="E128" s="488"/>
+      <c r="C128" s="514"/>
+      <c r="D128" s="515"/>
+      <c r="E128" s="515"/>
       <c r="G128" s="22"/>
       <c r="H128" s="22"/>
       <c r="I128" s="22"/>
@@ -16259,86 +16259,6 @@
     </row>
   </sheetData>
   <mergeCells count="96">
-    <mergeCell ref="A41:E41"/>
-    <mergeCell ref="A24:E24"/>
-    <mergeCell ref="A33:E33"/>
-    <mergeCell ref="C64:E64"/>
-    <mergeCell ref="A40:E40"/>
-    <mergeCell ref="A49:E49"/>
-    <mergeCell ref="C61:E61"/>
-    <mergeCell ref="A59:E59"/>
-    <mergeCell ref="C60:E60"/>
-    <mergeCell ref="A48:E48"/>
-    <mergeCell ref="C62:E62"/>
-    <mergeCell ref="C63:E63"/>
-    <mergeCell ref="A32:E32"/>
-    <mergeCell ref="C65:E65"/>
-    <mergeCell ref="A56:E58"/>
-    <mergeCell ref="C78:E78"/>
-    <mergeCell ref="C73:E73"/>
-    <mergeCell ref="C75:E75"/>
-    <mergeCell ref="C76:E76"/>
-    <mergeCell ref="C69:E69"/>
-    <mergeCell ref="C68:E68"/>
-    <mergeCell ref="C79:E79"/>
-    <mergeCell ref="C80:E80"/>
-    <mergeCell ref="C66:E66"/>
-    <mergeCell ref="C74:E74"/>
-    <mergeCell ref="C77:E77"/>
-    <mergeCell ref="C71:E71"/>
-    <mergeCell ref="C72:E72"/>
-    <mergeCell ref="C67:E67"/>
-    <mergeCell ref="C70:E70"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="A16:E17"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B20:D20"/>
-    <mergeCell ref="A25:E25"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="A18:E18"/>
-    <mergeCell ref="A19:E19"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="C105:E105"/>
-    <mergeCell ref="C98:E98"/>
-    <mergeCell ref="C81:E81"/>
-    <mergeCell ref="C82:E82"/>
-    <mergeCell ref="C83:E83"/>
-    <mergeCell ref="C89:E89"/>
-    <mergeCell ref="A94:E94"/>
-    <mergeCell ref="C96:E96"/>
-    <mergeCell ref="C86:E86"/>
-    <mergeCell ref="C87:E87"/>
-    <mergeCell ref="C85:E85"/>
-    <mergeCell ref="C95:E95"/>
-    <mergeCell ref="C88:E88"/>
-    <mergeCell ref="C84:E84"/>
-    <mergeCell ref="C104:E104"/>
-    <mergeCell ref="C121:E121"/>
-    <mergeCell ref="C122:E122"/>
-    <mergeCell ref="C110:E110"/>
-    <mergeCell ref="C111:E111"/>
-    <mergeCell ref="C106:E106"/>
-    <mergeCell ref="C107:E107"/>
-    <mergeCell ref="C108:E108"/>
-    <mergeCell ref="C128:E128"/>
-    <mergeCell ref="A124:E124"/>
-    <mergeCell ref="C125:E125"/>
-    <mergeCell ref="C126:E126"/>
-    <mergeCell ref="C127:E127"/>
     <mergeCell ref="I95:M95"/>
     <mergeCell ref="C119:E119"/>
     <mergeCell ref="A115:E115"/>
@@ -16355,6 +16275,86 @@
     <mergeCell ref="C101:E101"/>
     <mergeCell ref="C102:E102"/>
     <mergeCell ref="C103:E103"/>
+    <mergeCell ref="C128:E128"/>
+    <mergeCell ref="A124:E124"/>
+    <mergeCell ref="C125:E125"/>
+    <mergeCell ref="C126:E126"/>
+    <mergeCell ref="C127:E127"/>
+    <mergeCell ref="C121:E121"/>
+    <mergeCell ref="C122:E122"/>
+    <mergeCell ref="C110:E110"/>
+    <mergeCell ref="C111:E111"/>
+    <mergeCell ref="C106:E106"/>
+    <mergeCell ref="C107:E107"/>
+    <mergeCell ref="C108:E108"/>
+    <mergeCell ref="C105:E105"/>
+    <mergeCell ref="C98:E98"/>
+    <mergeCell ref="C81:E81"/>
+    <mergeCell ref="C82:E82"/>
+    <mergeCell ref="C83:E83"/>
+    <mergeCell ref="C89:E89"/>
+    <mergeCell ref="A94:E94"/>
+    <mergeCell ref="C96:E96"/>
+    <mergeCell ref="C86:E86"/>
+    <mergeCell ref="C87:E87"/>
+    <mergeCell ref="C85:E85"/>
+    <mergeCell ref="C95:E95"/>
+    <mergeCell ref="C88:E88"/>
+    <mergeCell ref="C84:E84"/>
+    <mergeCell ref="C104:E104"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="A16:E17"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="C79:E79"/>
+    <mergeCell ref="C80:E80"/>
+    <mergeCell ref="C66:E66"/>
+    <mergeCell ref="C74:E74"/>
+    <mergeCell ref="C77:E77"/>
+    <mergeCell ref="C71:E71"/>
+    <mergeCell ref="C72:E72"/>
+    <mergeCell ref="C67:E67"/>
+    <mergeCell ref="C70:E70"/>
+    <mergeCell ref="C65:E65"/>
+    <mergeCell ref="A56:E58"/>
+    <mergeCell ref="C78:E78"/>
+    <mergeCell ref="C73:E73"/>
+    <mergeCell ref="C75:E75"/>
+    <mergeCell ref="C76:E76"/>
+    <mergeCell ref="C69:E69"/>
+    <mergeCell ref="C68:E68"/>
+    <mergeCell ref="A41:E41"/>
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="A33:E33"/>
+    <mergeCell ref="C64:E64"/>
+    <mergeCell ref="A40:E40"/>
+    <mergeCell ref="A49:E49"/>
+    <mergeCell ref="C61:E61"/>
+    <mergeCell ref="A59:E59"/>
+    <mergeCell ref="C60:E60"/>
+    <mergeCell ref="A48:E48"/>
+    <mergeCell ref="C62:E62"/>
+    <mergeCell ref="C63:E63"/>
+    <mergeCell ref="A32:E32"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.39" right="0.26" top="0.66" bottom="0.71" header="0.5" footer="0.5"/>
@@ -16365,8 +16365,133 @@
   <controls>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="6150" r:id="rId4" name="TestDBConnection">
+        <control shapeId="6162" r:id="rId4" name="RiskModelManual">
           <controlPr defaultSize="0" autoLine="0" autoPict="0" r:id="rId5">
+            <anchor moveWithCells="1">
+              <from>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>2667000</xdr:colOff>
+                <xdr:row>14</xdr:row>
+                <xdr:rowOff>19050</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>3286125</xdr:colOff>
+                <xdr:row>15</xdr:row>
+                <xdr:rowOff>0</xdr:rowOff>
+              </to>
+            </anchor>
+          </controlPr>
+        </control>
+      </mc:Choice>
+      <mc:Fallback>
+        <control shapeId="6162" r:id="rId4" name="RiskModelManual"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <control shapeId="6161" r:id="rId6" name="RiskModelStandard">
+          <controlPr defaultSize="0" autoLine="0" r:id="rId7">
+            <anchor moveWithCells="1">
+              <from>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>1905000</xdr:colOff>
+                <xdr:row>14</xdr:row>
+                <xdr:rowOff>19050</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>2619375</xdr:colOff>
+                <xdr:row>15</xdr:row>
+                <xdr:rowOff>0</xdr:rowOff>
+              </to>
+            </anchor>
+          </controlPr>
+        </control>
+      </mc:Choice>
+      <mc:Fallback>
+        <control shapeId="6161" r:id="rId6" name="RiskModelStandard"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <control shapeId="6159" r:id="rId8" name="Auth_Custom">
+          <controlPr defaultSize="0" autoLine="0" r:id="rId9">
+            <anchor moveWithCells="1" sizeWithCells="1">
+              <from>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>1133475</xdr:colOff>
+                <xdr:row>125</xdr:row>
+                <xdr:rowOff>19050</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>2028825</xdr:colOff>
+                <xdr:row>125</xdr:row>
+                <xdr:rowOff>209550</xdr:rowOff>
+              </to>
+            </anchor>
+          </controlPr>
+        </control>
+      </mc:Choice>
+      <mc:Fallback>
+        <control shapeId="6159" r:id="rId8" name="Auth_Custom"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <control shapeId="6148" r:id="rId10" name="Auth_DB">
+          <controlPr defaultSize="0" autoLine="0" r:id="rId11">
+            <anchor moveWithCells="1" sizeWithCells="1">
+              <from>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>590550</xdr:colOff>
+                <xdr:row>125</xdr:row>
+                <xdr:rowOff>9525</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>1143000</xdr:colOff>
+                <xdr:row>125</xdr:row>
+                <xdr:rowOff>200025</xdr:rowOff>
+              </to>
+            </anchor>
+          </controlPr>
+        </control>
+      </mc:Choice>
+      <mc:Fallback>
+        <control shapeId="6148" r:id="rId10" name="Auth_DB"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <control shapeId="6146" r:id="rId12" name="Auth_NT">
+          <controlPr defaultSize="0" autoLine="0" autoPict="0" r:id="rId13">
+            <anchor moveWithCells="1" sizeWithCells="1">
+              <from>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>9525</xdr:colOff>
+                <xdr:row>125</xdr:row>
+                <xdr:rowOff>19050</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>600075</xdr:colOff>
+                <xdr:row>125</xdr:row>
+                <xdr:rowOff>200025</xdr:rowOff>
+              </to>
+            </anchor>
+          </controlPr>
+        </control>
+      </mc:Choice>
+      <mc:Fallback>
+        <control shapeId="6146" r:id="rId12" name="Auth_NT"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <control shapeId="6150" r:id="rId14" name="TestDBConnection">
+          <controlPr defaultSize="0" autoLine="0" autoPict="0" r:id="rId15">
             <anchor moveWithCells="1" sizeWithCells="1">
               <from>
                 <xdr:col>2</xdr:col>
@@ -16385,132 +16510,7 @@
         </control>
       </mc:Choice>
       <mc:Fallback>
-        <control shapeId="6150" r:id="rId4" name="TestDBConnection"/>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice Requires="x14">
-        <control shapeId="6146" r:id="rId6" name="Auth_NT">
-          <controlPr defaultSize="0" autoLine="0" autoPict="0" r:id="rId7">
-            <anchor moveWithCells="1" sizeWithCells="1">
-              <from>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>9525</xdr:colOff>
-                <xdr:row>125</xdr:row>
-                <xdr:rowOff>19050</xdr:rowOff>
-              </from>
-              <to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>600075</xdr:colOff>
-                <xdr:row>125</xdr:row>
-                <xdr:rowOff>200025</xdr:rowOff>
-              </to>
-            </anchor>
-          </controlPr>
-        </control>
-      </mc:Choice>
-      <mc:Fallback>
-        <control shapeId="6146" r:id="rId6" name="Auth_NT"/>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice Requires="x14">
-        <control shapeId="6148" r:id="rId8" name="Auth_DB">
-          <controlPr defaultSize="0" autoLine="0" r:id="rId9">
-            <anchor moveWithCells="1" sizeWithCells="1">
-              <from>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>590550</xdr:colOff>
-                <xdr:row>125</xdr:row>
-                <xdr:rowOff>9525</xdr:rowOff>
-              </from>
-              <to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>1143000</xdr:colOff>
-                <xdr:row>125</xdr:row>
-                <xdr:rowOff>200025</xdr:rowOff>
-              </to>
-            </anchor>
-          </controlPr>
-        </control>
-      </mc:Choice>
-      <mc:Fallback>
-        <control shapeId="6148" r:id="rId8" name="Auth_DB"/>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice Requires="x14">
-        <control shapeId="6159" r:id="rId10" name="Auth_Custom">
-          <controlPr defaultSize="0" autoLine="0" r:id="rId11">
-            <anchor moveWithCells="1" sizeWithCells="1">
-              <from>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>1133475</xdr:colOff>
-                <xdr:row>125</xdr:row>
-                <xdr:rowOff>19050</xdr:rowOff>
-              </from>
-              <to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>2028825</xdr:colOff>
-                <xdr:row>125</xdr:row>
-                <xdr:rowOff>209550</xdr:rowOff>
-              </to>
-            </anchor>
-          </controlPr>
-        </control>
-      </mc:Choice>
-      <mc:Fallback>
-        <control shapeId="6159" r:id="rId10" name="Auth_Custom"/>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice Requires="x14">
-        <control shapeId="6161" r:id="rId12" name="RiskModelStandard">
-          <controlPr defaultSize="0" autoLine="0" r:id="rId13">
-            <anchor moveWithCells="1">
-              <from>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>1905000</xdr:colOff>
-                <xdr:row>14</xdr:row>
-                <xdr:rowOff>19050</xdr:rowOff>
-              </from>
-              <to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>2619375</xdr:colOff>
-                <xdr:row>15</xdr:row>
-                <xdr:rowOff>0</xdr:rowOff>
-              </to>
-            </anchor>
-          </controlPr>
-        </control>
-      </mc:Choice>
-      <mc:Fallback>
-        <control shapeId="6161" r:id="rId12" name="RiskModelStandard"/>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice Requires="x14">
-        <control shapeId="6162" r:id="rId14" name="RiskModelManual">
-          <controlPr defaultSize="0" autoLine="0" autoPict="0" r:id="rId15">
-            <anchor moveWithCells="1">
-              <from>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>2667000</xdr:colOff>
-                <xdr:row>14</xdr:row>
-                <xdr:rowOff>19050</xdr:rowOff>
-              </from>
-              <to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>3286125</xdr:colOff>
-                <xdr:row>15</xdr:row>
-                <xdr:rowOff>0</xdr:rowOff>
-              </to>
-            </anchor>
-          </controlPr>
-        </control>
-      </mc:Choice>
-      <mc:Fallback>
-        <control shapeId="6162" r:id="rId14" name="RiskModelManual"/>
+        <control shapeId="6150" r:id="rId14" name="TestDBConnection"/>
       </mc:Fallback>
     </mc:AlternateContent>
   </controls>
@@ -16602,7 +16602,7 @@
       <c r="B4" s="40" t="s">
         <v>75</v>
       </c>
-      <c r="C4" s="455" t="s">
+      <c r="C4" s="458" t="s">
         <v>187</v>
       </c>
       <c r="D4" s="521"/>
@@ -16791,12 +16791,12 @@
       <c r="B16" s="40" t="s">
         <v>75</v>
       </c>
-      <c r="C16" s="528" t="s">
+      <c r="C16" s="545" t="s">
         <v>201</v>
       </c>
-      <c r="D16" s="529"/>
-      <c r="E16" s="530"/>
-      <c r="F16" s="531"/>
+      <c r="D16" s="546"/>
+      <c r="E16" s="547"/>
+      <c r="F16" s="548"/>
       <c r="G16" s="41"/>
       <c r="H16" s="41"/>
       <c r="I16" s="41"/>
@@ -16961,12 +16961,12 @@
       <c r="B27" s="204" t="s">
         <v>75</v>
       </c>
-      <c r="C27" s="528" t="s">
+      <c r="C27" s="545" t="s">
         <v>425</v>
       </c>
-      <c r="D27" s="529"/>
-      <c r="E27" s="530"/>
-      <c r="F27" s="531"/>
+      <c r="D27" s="546"/>
+      <c r="E27" s="547"/>
+      <c r="F27" s="548"/>
       <c r="G27" s="41"/>
       <c r="H27" s="41"/>
       <c r="I27" s="41"/>
@@ -17129,14 +17129,14 @@
       <c r="B40" s="231" t="s">
         <v>62</v>
       </c>
-      <c r="C40" s="532" t="s">
+      <c r="C40" s="549" t="s">
         <v>61</v>
       </c>
-      <c r="D40" s="533"/>
-      <c r="E40" s="534" t="s">
+      <c r="D40" s="550"/>
+      <c r="E40" s="551" t="s">
         <v>185</v>
       </c>
-      <c r="F40" s="535"/>
+      <c r="F40" s="552"/>
       <c r="G40" s="232" t="s">
         <v>174</v>
       </c>
@@ -17154,12 +17154,12 @@
       <c r="B41" s="234" t="s">
         <v>75</v>
       </c>
-      <c r="C41" s="524" t="s">
+      <c r="C41" s="541" t="s">
         <v>187</v>
       </c>
-      <c r="D41" s="525"/>
-      <c r="E41" s="526"/>
-      <c r="F41" s="527"/>
+      <c r="D41" s="542"/>
+      <c r="E41" s="543"/>
+      <c r="F41" s="544"/>
       <c r="G41" s="235"/>
       <c r="H41" s="235"/>
       <c r="I41" s="235"/>
@@ -17300,30 +17300,30 @@
     </row>
     <row r="52" spans="1:9" ht="13.5" thickBot="1"/>
     <row r="53" spans="1:9" ht="30" customHeight="1">
-      <c r="A53" s="536" t="s">
+      <c r="A53" s="524" t="s">
         <v>212</v>
       </c>
-      <c r="B53" s="537"/>
-      <c r="C53" s="538"/>
-      <c r="D53" s="539"/>
-      <c r="E53" s="540"/>
-      <c r="F53" s="540"/>
-      <c r="G53" s="540"/>
-      <c r="H53" s="467"/>
-      <c r="I53" s="541"/>
+      <c r="B53" s="525"/>
+      <c r="C53" s="526"/>
+      <c r="D53" s="527"/>
+      <c r="E53" s="528"/>
+      <c r="F53" s="528"/>
+      <c r="G53" s="528"/>
+      <c r="H53" s="466"/>
+      <c r="I53" s="529"/>
     </row>
     <row r="54" spans="1:9" ht="30" customHeight="1" thickBot="1">
-      <c r="A54" s="542" t="s">
+      <c r="A54" s="530" t="s">
         <v>42</v>
       </c>
-      <c r="B54" s="543"/>
-      <c r="C54" s="544"/>
-      <c r="D54" s="545"/>
-      <c r="E54" s="546"/>
-      <c r="F54" s="546"/>
-      <c r="G54" s="546"/>
-      <c r="H54" s="547"/>
-      <c r="I54" s="548"/>
+      <c r="B54" s="531"/>
+      <c r="C54" s="532"/>
+      <c r="D54" s="533"/>
+      <c r="E54" s="534"/>
+      <c r="F54" s="534"/>
+      <c r="G54" s="534"/>
+      <c r="H54" s="535"/>
+      <c r="I54" s="536"/>
     </row>
     <row r="55" spans="1:9" ht="31.5">
       <c r="A55" s="126" t="s">
@@ -17332,14 +17332,14 @@
       <c r="B55" s="121" t="s">
         <v>62</v>
       </c>
-      <c r="C55" s="549" t="s">
+      <c r="C55" s="537" t="s">
         <v>61</v>
       </c>
-      <c r="D55" s="550"/>
-      <c r="E55" s="551" t="s">
+      <c r="D55" s="538"/>
+      <c r="E55" s="539" t="s">
         <v>185</v>
       </c>
-      <c r="F55" s="552"/>
+      <c r="F55" s="540"/>
       <c r="G55" s="122" t="s">
         <v>174</v>
       </c>
@@ -17353,7 +17353,7 @@
     <row r="56" spans="1:9" ht="39" customHeight="1" thickBot="1">
       <c r="A56" s="118"/>
       <c r="B56" s="125"/>
-      <c r="C56" s="455"/>
+      <c r="C56" s="458"/>
       <c r="D56" s="521"/>
       <c r="E56" s="522"/>
       <c r="F56" s="523"/>
@@ -17384,14 +17384,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="C56:D56"/>
-    <mergeCell ref="E56:F56"/>
-    <mergeCell ref="A53:C53"/>
-    <mergeCell ref="D53:I53"/>
-    <mergeCell ref="A54:C54"/>
-    <mergeCell ref="D54:I54"/>
-    <mergeCell ref="C55:D55"/>
-    <mergeCell ref="E55:F55"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="C41:D41"/>
@@ -17402,6 +17394,14 @@
     <mergeCell ref="E40:F40"/>
     <mergeCell ref="C27:D27"/>
     <mergeCell ref="E27:F27"/>
+    <mergeCell ref="C56:D56"/>
+    <mergeCell ref="E56:F56"/>
+    <mergeCell ref="A53:C53"/>
+    <mergeCell ref="D53:I53"/>
+    <mergeCell ref="A54:C54"/>
+    <mergeCell ref="D54:I54"/>
+    <mergeCell ref="C55:D55"/>
+    <mergeCell ref="E55:F55"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.36" right="0.55000000000000004" top="0.61" bottom="0.62" header="0.36" footer="0.39"/>
@@ -19914,18 +19914,18 @@
   <controls>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="219440" r:id="rId4" name="Btn_Insert">
+        <control shapeId="219442" r:id="rId4" name="Btn_Duplicate">
           <controlPr defaultSize="0" print="0" autoLine="0" r:id="rId5">
             <anchor>
               <from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>104775</xdr:colOff>
+                <xdr:col>5</xdr:col>
+                <xdr:colOff>457200</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>28575</xdr:rowOff>
               </from>
               <to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>657225</xdr:colOff>
+                <xdr:col>6</xdr:col>
+                <xdr:colOff>971550</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>381000</xdr:rowOff>
               </to>
@@ -19934,7 +19934,7 @@
         </control>
       </mc:Choice>
       <mc:Fallback>
-        <control shapeId="219440" r:id="rId4" name="Btn_Insert"/>
+        <control shapeId="219442" r:id="rId4" name="Btn_Duplicate"/>
       </mc:Fallback>
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -19964,18 +19964,18 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="219442" r:id="rId8" name="Btn_Duplicate">
+        <control shapeId="219440" r:id="rId8" name="Btn_Insert">
           <controlPr defaultSize="0" print="0" autoLine="0" r:id="rId9">
             <anchor>
               <from>
-                <xdr:col>5</xdr:col>
-                <xdr:colOff>457200</xdr:colOff>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>104775</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>28575</xdr:rowOff>
               </from>
               <to>
-                <xdr:col>6</xdr:col>
-                <xdr:colOff>971550</xdr:colOff>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>657225</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>381000</xdr:rowOff>
               </to>
@@ -19984,7 +19984,7 @@
         </control>
       </mc:Choice>
       <mc:Fallback>
-        <control shapeId="219442" r:id="rId8" name="Btn_Duplicate"/>
+        <control shapeId="219440" r:id="rId8" name="Btn_Insert"/>
       </mc:Fallback>
     </mc:AlternateContent>
   </controls>
@@ -20902,18 +20902,18 @@
   <controls>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="451585" r:id="rId4" name="Btn_Insert">
+        <control shapeId="451587" r:id="rId4" name="Btn_Duplicate">
           <controlPr defaultSize="0" autoLine="0" r:id="rId5">
             <anchor moveWithCells="1">
               <from>
-                <xdr:col>4</xdr:col>
-                <xdr:colOff>133350</xdr:colOff>
+                <xdr:col>6</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>28575</xdr:rowOff>
               </from>
               <to>
-                <xdr:col>5</xdr:col>
-                <xdr:colOff>114300</xdr:colOff>
+                <xdr:col>7</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>381000</xdr:rowOff>
               </to>
@@ -20922,7 +20922,7 @@
         </control>
       </mc:Choice>
       <mc:Fallback>
-        <control shapeId="451585" r:id="rId4" name="Btn_Insert"/>
+        <control shapeId="451587" r:id="rId4" name="Btn_Duplicate"/>
       </mc:Fallback>
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -20952,18 +20952,18 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="451587" r:id="rId8" name="Btn_Duplicate">
+        <control shapeId="451585" r:id="rId8" name="Btn_Insert">
           <controlPr defaultSize="0" autoLine="0" r:id="rId9">
             <anchor moveWithCells="1">
               <from>
-                <xdr:col>6</xdr:col>
-                <xdr:colOff>0</xdr:colOff>
+                <xdr:col>4</xdr:col>
+                <xdr:colOff>133350</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>28575</xdr:rowOff>
               </from>
               <to>
-                <xdr:col>7</xdr:col>
-                <xdr:colOff>0</xdr:colOff>
+                <xdr:col>5</xdr:col>
+                <xdr:colOff>114300</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>381000</xdr:rowOff>
               </to>
@@ -20972,7 +20972,7 @@
         </control>
       </mc:Choice>
       <mc:Fallback>
-        <control shapeId="451587" r:id="rId8" name="Btn_Duplicate"/>
+        <control shapeId="451585" r:id="rId8" name="Btn_Insert"/>
       </mc:Fallback>
     </mc:AlternateContent>
   </controls>
@@ -21154,15 +21154,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101001D22062C56AC5E408EE4AD716EF9D51F" ma:contentTypeVersion="2" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="ea406ecd760878d0eb1cc59d2f82b96a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9345d9e0-45ad-4592-a016-571b7fc0fa4f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2786b7ba02371c72a8121ab12a0a4c41" ns2:_="">
     <xsd:import namespace="9345d9e0-45ad-4592-a016-571b7fc0fa4f"/>
@@ -21294,6 +21285,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FEE12B09-4783-40EA-8AF6-8843BC80EF2E}">
   <ds:schemaRefs>
@@ -21311,14 +21311,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4690AC4-6964-43EF-B841-F7D846FC4414}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B82E831-EF78-42F1-BD6A-915864E05434}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -21334,4 +21326,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4690AC4-6964-43EF-B841-F7D846FC4414}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>